<commit_message>
Schedule web Wi-Fi management (R-37) in Jacky's dev and test items.
Seven items in W4 (11/2-11/6): firmware add/remove/report and scan,
voice-server relay with an owner check and no stored passwords, the
settings page, and three tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project-schedule.xlsx
+++ b/docs/project-schedule.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="變更記錄" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Jacky 開發與測試'!$A$6:$M$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Jacky 開發與測試'!$A$6:$M$117</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Jacky 開發與測試'!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1638,7 +1638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M115"/>
+  <dimension ref="A1:M122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1672,26 +1672,26 @@
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="17">
-        <f>"開發項目：已完成 "&amp;COUNTIFS($B$7:$B$110,"開發",$J$7:$J$110,"已完成")&amp;" / "&amp;COUNTIF($B$7:$B$110,"開發")</f>
+        <f>"開發項目：已完成 "&amp;COUNTIFS($B$7:$B$117,"開發",$J$7:$J$117,"已完成")&amp;" / "&amp;COUNTIF($B$7:$B$117,"開發")</f>
         <v/>
       </c>
       <c r="B4" s="18" t="n"/>
       <c r="C4" s="18" t="n"/>
       <c r="D4" s="19" t="n"/>
       <c r="E4" s="17">
-        <f>"測試項目：已完成 "&amp;COUNTIFS($B$7:$B$110,"測試",$J$7:$J$110,"已完成")&amp;" / "&amp;COUNTIF($B$7:$B$110,"測試")</f>
+        <f>"測試項目：已完成 "&amp;COUNTIFS($B$7:$B$117,"測試",$J$7:$J$117,"已完成")&amp;" / "&amp;COUNTIF($B$7:$B$117,"測試")</f>
         <v/>
       </c>
       <c r="F4" s="18" t="n"/>
       <c r="G4" s="19" t="n"/>
       <c r="H4" s="17">
-        <f>"逾期未完成："&amp;COUNTIF($L$7:$L$110,"&gt;0")</f>
+        <f>"逾期未完成："&amp;COUNTIF($L$7:$L$117,"&gt;0")</f>
         <v/>
       </c>
       <c r="I4" s="18" t="n"/>
       <c r="J4" s="19" t="n"/>
       <c r="K4" s="17">
-        <f>"本週到期未完成："&amp;COUNTIFS($F$7:$F$110,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),$F$7:$F$110,"&lt;="&amp;((TODAY()-WEEKDAY(TODAY(),3))+6),$J$7:$J$110,"&lt;&gt;已完成")</f>
+        <f>"本週到期未完成："&amp;COUNTIFS($F$7:$F$117,"&gt;="&amp;(TODAY()-WEEKDAY(TODAY(),3)),$F$7:$F$117,"&lt;="&amp;((TODAY()-WEEKDAY(TODAY(),3))+6),$J$7:$J$117,"&lt;&gt;已完成")</f>
         <v/>
       </c>
       <c r="L4" s="18" t="n"/>
@@ -3648,7 +3648,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="34" customHeight="1">
+    <row r="43" ht="49" customHeight="1">
       <c r="A43" s="20" t="n">
         <v>37</v>
       </c>
@@ -3659,26 +3659,30 @@
       </c>
       <c r="C43" s="21" t="inlineStr">
         <is>
-          <t>RAG 知識庫（快活）</t>
+          <t>網頁：Wi-Fi 管理</t>
         </is>
       </c>
       <c r="D43" s="21" t="inlineStr">
         <is>
-          <t>知識庫的資料表、入庫腳本、版本和審批欄位</t>
+          <t>韌體：經連線接收新增、刪除 Wi-Fi；回報已記住的清單、目前 Wi-Fi 和訊號；上限加到 8 個</t>
         </is>
       </c>
       <c r="E43" s="22" t="n">
         <v>46328</v>
       </c>
       <c r="F43" s="22" t="n">
-        <v>46330</v>
+        <v>46329</v>
       </c>
       <c r="G43" s="21" t="inlineStr">
         <is>
-          <t>可以上載、送審、批准；只有批准的版本會被使用</t>
-        </is>
-      </c>
-      <c r="H43" s="21" t="inlineStr"/>
+          <t>網頁送出後玩具即時更新清單；重新開機後清單不變</t>
+        </is>
+      </c>
+      <c r="H43" s="21" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
       <c r="I43" s="21" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -3694,7 +3698,11 @@
         <f>IF(J43="已完成",IF(K43="","",MAX(0,K43-F43)),IF(TODAY()&gt;F43,TODAY()-F43,""))</f>
         <v/>
       </c>
-      <c r="M43" s="21" t="inlineStr"/>
+      <c r="M43" s="21" t="inlineStr">
+        <is>
+          <t>經 OTA 推出</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="34" customHeight="1">
       <c r="A44" s="23" t="n">
@@ -3707,26 +3715,30 @@
       </c>
       <c r="C44" s="24" t="inlineStr">
         <is>
-          <t>RAG 知識庫（快活）</t>
+          <t>網頁：Wi-Fi 管理</t>
         </is>
       </c>
       <c r="D44" s="24" t="inlineStr">
         <is>
-          <t>把馬會第一批資料入庫</t>
+          <t>韌體：待機時掃描附近 Wi-Fi，回傳清單</t>
         </is>
       </c>
       <c r="E44" s="25" t="n">
-        <v>46331</v>
+        <v>46329</v>
       </c>
       <c r="F44" s="25" t="n">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="G44" s="24" t="inlineStr">
         <is>
-          <t>Navy 整理的問答全部入庫</t>
-        </is>
-      </c>
-      <c r="H44" s="24" t="inlineStr"/>
+          <t>掃描不影響對話（只在待機時掃）</t>
+        </is>
+      </c>
+      <c r="H44" s="24" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
       <c r="I44" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -3742,43 +3754,43 @@
         <f>IF(J44="已完成",IF(K44="","",MAX(0,K44-F44)),IF(TODAY()&gt;F44,TODAY()-F44,""))</f>
         <v/>
       </c>
-      <c r="M44" s="24" t="inlineStr">
-        <is>
-          <t>要等馬會交資料</t>
-        </is>
-      </c>
+      <c r="M44" s="24" t="inlineStr"/>
     </row>
     <row r="45" ht="34" customHeight="1">
       <c r="A45" s="23" t="n">
         <v>39</v>
       </c>
-      <c r="B45" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
+      <c r="B45" s="23" t="inlineStr">
+        <is>
+          <t>開發</t>
         </is>
       </c>
       <c r="C45" s="24" t="inlineStr">
         <is>
-          <t>RAG 知識庫（快活）</t>
+          <t>網頁：Wi-Fi 管理</t>
         </is>
       </c>
       <c r="D45" s="24" t="inlineStr">
         <is>
-          <t>入庫 → 送審 → 批准 → 生效，跑一次</t>
+          <t>語音伺服器：確認是設備主人後轉送；密碼不寫入資料庫和日誌</t>
         </is>
       </c>
       <c r="E45" s="25" t="n">
-        <v>46332</v>
+        <v>46329</v>
       </c>
       <c r="F45" s="25" t="n">
-        <v>46332</v>
+        <v>46330</v>
       </c>
       <c r="G45" s="24" t="inlineStr">
         <is>
-          <t>流程跑通；未批准的內容不會被回答使用</t>
-        </is>
-      </c>
-      <c r="H45" s="24" t="inlineStr"/>
+          <t>非主人呼叫回 403</t>
+        </is>
+      </c>
+      <c r="H45" s="24" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
       <c r="I45" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -3807,26 +3819,30 @@
       </c>
       <c r="C46" s="24" t="inlineStr">
         <is>
-          <t>RAG 知識庫（快活）</t>
+          <t>網頁：Wi-Fi 管理</t>
         </is>
       </c>
       <c r="D46" s="24" t="inlineStr">
         <is>
-          <t>對話時檢索知識庫並回答</t>
+          <t>設定頁：在線狀態、目前 Wi-Fi、我的 Wi-Fi、新增、刪除</t>
         </is>
       </c>
       <c r="E46" s="25" t="n">
-        <v>46335</v>
+        <v>46330</v>
       </c>
       <c r="F46" s="25" t="n">
-        <v>46346</v>
+        <v>46332</v>
       </c>
       <c r="G46" s="24" t="inlineStr">
         <is>
-          <t>問到知識庫的內容時，回答引用知識庫</t>
-        </is>
-      </c>
-      <c r="H46" s="24" t="inlineStr"/>
+          <t>對照參考圖；不能刪除正在使用的 Wi-Fi；離線時新增按鈕停用</t>
+        </is>
+      </c>
+      <c r="H46" s="24" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
       <c r="I46" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -3842,39 +3858,47 @@
         <f>IF(J46="已完成",IF(K46="","",MAX(0,K46-F46)),IF(TODAY()&gt;F46,TODAY()-F46,""))</f>
         <v/>
       </c>
-      <c r="M46" s="24" t="inlineStr"/>
+      <c r="M46" s="24" t="inlineStr">
+        <is>
+          <t>Navy 的設計稿到了再換外觀</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="34" customHeight="1">
       <c r="A47" s="23" t="n">
         <v>41</v>
       </c>
-      <c r="B47" s="23" t="inlineStr">
-        <is>
-          <t>開發</t>
+      <c r="B47" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
         </is>
       </c>
       <c r="C47" s="24" t="inlineStr">
         <is>
-          <t>RAG 知識庫（快活）</t>
+          <t>網頁：Wi-Fi 管理</t>
         </is>
       </c>
       <c r="D47" s="24" t="inlineStr">
         <is>
-          <t>沒把握時的說法；婉拒貼士、賠率、賽果預測</t>
+          <t>網頁新增 Wi-Fi B，然後關掉原來的 Wi-Fi A</t>
         </is>
       </c>
       <c r="E47" s="25" t="n">
-        <v>46344</v>
+        <v>46332</v>
       </c>
       <c r="F47" s="25" t="n">
-        <v>46350</v>
+        <v>46332</v>
       </c>
       <c r="G47" s="24" t="inlineStr">
         <is>
-          <t>知識庫沒有的內容會說不肯定並建議查詢</t>
-        </is>
-      </c>
-      <c r="H47" s="24" t="inlineStr"/>
+          <t>玩具自動改連 B</t>
+        </is>
+      </c>
+      <c r="H47" s="24" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
       <c r="I47" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -3896,33 +3920,37 @@
       <c r="A48" s="23" t="n">
         <v>42</v>
       </c>
-      <c r="B48" s="23" t="inlineStr">
-        <is>
-          <t>開發</t>
+      <c r="B48" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
         </is>
       </c>
       <c r="C48" s="24" t="inlineStr">
         <is>
-          <t>RAG 知識庫（快活）</t>
+          <t>網頁：Wi-Fi 管理</t>
         </is>
       </c>
       <c r="D48" s="24" t="inlineStr">
         <is>
-          <t>測試問題自動跑分的腳本</t>
+          <t>B 的密碼打錯；嘗試刪除目前 Wi-Fi；用另一個帳號呼叫</t>
         </is>
       </c>
       <c r="E48" s="25" t="n">
-        <v>46349</v>
+        <v>46332</v>
       </c>
       <c r="F48" s="25" t="n">
-        <v>46353</v>
+        <v>46332</v>
       </c>
       <c r="G48" s="24" t="inlineStr">
         <is>
-          <t>一條命令跑完 100 條問題並出分數</t>
-        </is>
-      </c>
-      <c r="H48" s="24" t="inlineStr"/>
+          <t>玩具留在 A 不斷線；刪除被拒；另一帳號 403</t>
+        </is>
+      </c>
+      <c r="H48" s="24" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
       <c r="I48" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -3938,11 +3966,7 @@
         <f>IF(J48="已完成",IF(K48="","",MAX(0,K48-F48)),IF(TODAY()&gt;F48,TODAY()-F48,""))</f>
         <v/>
       </c>
-      <c r="M48" s="24" t="inlineStr">
-        <is>
-          <t>Navy 寫問題和標準答案</t>
-        </is>
-      </c>
+      <c r="M48" s="24" t="inlineStr"/>
     </row>
     <row r="49" ht="34" customHeight="1">
       <c r="A49" s="23" t="n">
@@ -3955,26 +3979,30 @@
       </c>
       <c r="C49" s="24" t="inlineStr">
         <is>
-          <t>RAG 知識庫（快活）</t>
+          <t>網頁：Wi-Fi 管理</t>
         </is>
       </c>
       <c r="D49" s="24" t="inlineStr">
         <is>
-          <t>跑 100 條測試問題</t>
+          <t>搜尋資料庫和伺服器日誌裡的測試密碼</t>
         </is>
       </c>
       <c r="E49" s="25" t="n">
-        <v>46357</v>
+        <v>46332</v>
       </c>
       <c r="F49" s="25" t="n">
-        <v>46360</v>
+        <v>46332</v>
       </c>
       <c r="G49" s="24" t="inlineStr">
         <is>
-          <t>答對率 ≥ 80%</t>
-        </is>
-      </c>
-      <c r="H49" s="24" t="inlineStr"/>
+          <t>找不到</t>
+        </is>
+      </c>
+      <c r="H49" s="24" t="inlineStr">
+        <is>
+          <t>R-37</t>
+        </is>
+      </c>
       <c r="I49" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -3993,52 +4021,52 @@
       <c r="M49" s="24" t="inlineStr"/>
     </row>
     <row r="50" ht="34" customHeight="1">
-      <c r="A50" s="23" t="n">
+      <c r="A50" s="20" t="n">
         <v>44</v>
       </c>
-      <c r="B50" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
-        </is>
-      </c>
-      <c r="C50" s="24" t="inlineStr">
+      <c r="B50" s="20" t="inlineStr">
+        <is>
+          <t>開發</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
         <is>
           <t>RAG 知識庫（快活）</t>
         </is>
       </c>
-      <c r="D50" s="24" t="inlineStr">
-        <is>
-          <t>婉拒測試：至少 50 條問貼士、賠率、預測的問題，包括換說法和三種語言</t>
-        </is>
-      </c>
-      <c r="E50" s="25" t="n">
-        <v>46357</v>
-      </c>
-      <c r="F50" s="25" t="n">
-        <v>46360</v>
-      </c>
-      <c r="G50" s="24" t="inlineStr">
-        <is>
-          <t>100% 婉拒</t>
-        </is>
-      </c>
-      <c r="H50" s="24" t="inlineStr"/>
-      <c r="I50" s="24" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J50" s="23" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K50" s="25" t="n"/>
-      <c r="L50" s="23">
+      <c r="D50" s="21" t="inlineStr">
+        <is>
+          <t>知識庫的資料表、入庫腳本、版本和審批欄位</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="n">
+        <v>46328</v>
+      </c>
+      <c r="F50" s="22" t="n">
+        <v>46330</v>
+      </c>
+      <c r="G50" s="21" t="inlineStr">
+        <is>
+          <t>可以上載、送審、批准；只有批准的版本會被使用</t>
+        </is>
+      </c>
+      <c r="H50" s="21" t="inlineStr"/>
+      <c r="I50" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J50" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K50" s="22" t="n"/>
+      <c r="L50" s="20">
         <f>IF(J50="已完成",IF(K50="","",MAX(0,K50-F50)),IF(TODAY()&gt;F50,TODAY()-F50,""))</f>
         <v/>
       </c>
-      <c r="M50" s="24" t="inlineStr"/>
+      <c r="M50" s="21" t="inlineStr"/>
     </row>
     <row r="51" ht="34" customHeight="1">
       <c r="A51" s="23" t="n">
@@ -4056,18 +4084,18 @@
       </c>
       <c r="D51" s="24" t="inlineStr">
         <is>
-          <t>按馬會審核意見修改</t>
+          <t>把馬會第一批資料入庫</t>
         </is>
       </c>
       <c r="E51" s="25" t="n">
-        <v>46370</v>
+        <v>46331</v>
       </c>
       <c r="F51" s="25" t="n">
-        <v>46381</v>
+        <v>46332</v>
       </c>
       <c r="G51" s="24" t="inlineStr">
         <is>
-          <t>每次修改都有新版本和審批記錄</t>
+          <t>Navy 整理的問答全部入庫</t>
         </is>
       </c>
       <c r="H51" s="24" t="inlineStr"/>
@@ -4086,7 +4114,11 @@
         <f>IF(J51="已完成",IF(K51="","",MAX(0,K51-F51)),IF(TODAY()&gt;F51,TODAY()-F51,""))</f>
         <v/>
       </c>
-      <c r="M51" s="24" t="inlineStr"/>
+      <c r="M51" s="24" t="inlineStr">
+        <is>
+          <t>要等馬會交資料</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="34" customHeight="1">
       <c r="A52" s="23" t="n">
@@ -4104,18 +4136,18 @@
       </c>
       <c r="D52" s="24" t="inlineStr">
         <is>
-          <t>在後台更新知識庫，用已出廠的玩具提問</t>
+          <t>入庫 → 送審 → 批准 → 生效，跑一次</t>
         </is>
       </c>
       <c r="E52" s="25" t="n">
-        <v>46377</v>
+        <v>46332</v>
       </c>
       <c r="F52" s="25" t="n">
-        <v>46381</v>
+        <v>46332</v>
       </c>
       <c r="G52" s="24" t="inlineStr">
         <is>
-          <t>不用重新燒錄，玩具即時用新版本回答</t>
+          <t>流程跑通；未批准的內容不會被回答使用</t>
         </is>
       </c>
       <c r="H52" s="24" t="inlineStr"/>
@@ -4137,92 +4169,84 @@
       <c r="M52" s="24" t="inlineStr"/>
     </row>
     <row r="53" ht="34" customHeight="1">
-      <c r="A53" s="20" t="n">
+      <c r="A53" s="23" t="n">
         <v>47</v>
       </c>
-      <c r="B53" s="20" t="inlineStr">
+      <c r="B53" s="23" t="inlineStr">
         <is>
           <t>開發</t>
         </is>
       </c>
-      <c r="C53" s="21" t="inlineStr">
-        <is>
-          <t>韌體：分區表和加密</t>
-        </is>
-      </c>
-      <c r="D53" s="21" t="inlineStr">
-        <is>
-          <t>新分區表：加大 app 分區，加品牌資源分區和出廠設定分區</t>
-        </is>
-      </c>
-      <c r="E53" s="22" t="n">
-        <v>46314</v>
-      </c>
-      <c r="F53" s="22" t="n">
-        <v>46325</v>
-      </c>
-      <c r="G53" s="21" t="inlineStr">
-        <is>
-          <t>新分區表能放下現在的韌體加 30% 空間</t>
-        </is>
-      </c>
-      <c r="H53" s="21" t="inlineStr">
-        <is>
-          <t>P2-12</t>
-        </is>
-      </c>
-      <c r="I53" s="21" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J53" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K53" s="22" t="n"/>
-      <c r="L53" s="20">
+      <c r="C53" s="24" t="inlineStr">
+        <is>
+          <t>RAG 知識庫（快活）</t>
+        </is>
+      </c>
+      <c r="D53" s="24" t="inlineStr">
+        <is>
+          <t>對話時檢索知識庫並回答</t>
+        </is>
+      </c>
+      <c r="E53" s="25" t="n">
+        <v>46335</v>
+      </c>
+      <c r="F53" s="25" t="n">
+        <v>46346</v>
+      </c>
+      <c r="G53" s="24" t="inlineStr">
+        <is>
+          <t>問到知識庫的內容時，回答引用知識庫</t>
+        </is>
+      </c>
+      <c r="H53" s="24" t="inlineStr"/>
+      <c r="I53" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J53" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K53" s="25" t="n"/>
+      <c r="L53" s="23">
         <f>IF(J53="已完成",IF(K53="","",MAX(0,K53-F53)),IF(TODAY()&gt;F53,TODAY()-F53,""))</f>
         <v/>
       </c>
-      <c r="M53" s="21" t="inlineStr"/>
+      <c r="M53" s="24" t="inlineStr"/>
     </row>
     <row r="54" ht="34" customHeight="1">
       <c r="A54" s="23" t="n">
         <v>48</v>
       </c>
-      <c r="B54" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
+      <c r="B54" s="23" t="inlineStr">
+        <is>
+          <t>開發</t>
         </is>
       </c>
       <c r="C54" s="24" t="inlineStr">
         <is>
-          <t>韌體：分區表和加密</t>
+          <t>RAG 知識庫（快活）</t>
         </is>
       </c>
       <c r="D54" s="24" t="inlineStr">
         <is>
-          <t>新分區表上做 OTA 升級和回滾各一次</t>
+          <t>沒把握時的說法；婉拒貼士、賠率、賽果預測</t>
         </is>
       </c>
       <c r="E54" s="25" t="n">
-        <v>46328</v>
+        <v>46344</v>
       </c>
       <c r="F54" s="25" t="n">
-        <v>46330</v>
+        <v>46350</v>
       </c>
       <c r="G54" s="24" t="inlineStr">
         <is>
-          <t>兩次都成功</t>
-        </is>
-      </c>
-      <c r="H54" s="24" t="inlineStr">
-        <is>
-          <t>P2-12、P0-13</t>
-        </is>
-      </c>
+          <t>知識庫沒有的內容會說不肯定並建議查詢</t>
+        </is>
+      </c>
+      <c r="H54" s="24" t="inlineStr"/>
       <c r="I54" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -4251,30 +4275,26 @@
       </c>
       <c r="C55" s="24" t="inlineStr">
         <is>
-          <t>韌體：分區表和加密</t>
+          <t>RAG 知識庫（快活）</t>
         </is>
       </c>
       <c r="D55" s="24" t="inlineStr">
         <is>
-          <t>產生 Secure Boot 簽名金鑰，離線備份兩份</t>
+          <t>測試問題自動跑分的腳本</t>
         </is>
       </c>
       <c r="E55" s="25" t="n">
-        <v>46328</v>
+        <v>46349</v>
       </c>
       <c r="F55" s="25" t="n">
-        <v>46332</v>
+        <v>46353</v>
       </c>
       <c r="G55" s="24" t="inlineStr">
         <is>
-          <t>金鑰不在 repo、不在伺服器；備份放在兩個地方</t>
-        </is>
-      </c>
-      <c r="H55" s="24" t="inlineStr">
-        <is>
-          <t>P0-14</t>
-        </is>
-      </c>
+          <t>一條命令跑完 100 條問題並出分數</t>
+        </is>
+      </c>
+      <c r="H55" s="24" t="inlineStr"/>
       <c r="I55" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -4292,7 +4312,7 @@
       </c>
       <c r="M55" s="24" t="inlineStr">
         <is>
-          <t>金鑰遺失 = 所有玩具不能再 OTA</t>
+          <t>Navy 寫問題和標準答案</t>
         </is>
       </c>
     </row>
@@ -4300,37 +4320,33 @@
       <c r="A56" s="23" t="n">
         <v>50</v>
       </c>
-      <c r="B56" s="23" t="inlineStr">
-        <is>
-          <t>開發</t>
+      <c r="B56" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
         </is>
       </c>
       <c r="C56" s="24" t="inlineStr">
         <is>
-          <t>韌體：分區表和加密</t>
+          <t>RAG 知識庫（快活）</t>
         </is>
       </c>
       <c r="D56" s="24" t="inlineStr">
         <is>
-          <t>編譯流程加簽名和 Flash 加密</t>
+          <t>跑 100 條測試問題</t>
         </is>
       </c>
       <c r="E56" s="25" t="n">
-        <v>46330</v>
+        <v>46357</v>
       </c>
       <c r="F56" s="25" t="n">
-        <v>46336</v>
+        <v>46360</v>
       </c>
       <c r="G56" s="24" t="inlineStr">
         <is>
-          <t>一條命令出簽名後的正式映像</t>
-        </is>
-      </c>
-      <c r="H56" s="24" t="inlineStr">
-        <is>
-          <t>P0-14</t>
-        </is>
-      </c>
+          <t>答對率 ≥ 80%</t>
+        </is>
+      </c>
+      <c r="H56" s="24" t="inlineStr"/>
       <c r="I56" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -4359,30 +4375,26 @@
       </c>
       <c r="C57" s="24" t="inlineStr">
         <is>
-          <t>韌體：分區表和加密</t>
+          <t>RAG 知識庫（快活）</t>
         </is>
       </c>
       <c r="D57" s="24" t="inlineStr">
         <is>
-          <t>一片測試板燒 eFuse：簽名映像開機、未簽名映像 OTA、讀出 flash</t>
+          <t>婉拒測試：至少 50 條問貼士、賠率、預測的問題，包括換說法和三種語言</t>
         </is>
       </c>
       <c r="E57" s="25" t="n">
-        <v>46337</v>
+        <v>46357</v>
       </c>
       <c r="F57" s="25" t="n">
-        <v>46339</v>
+        <v>46360</v>
       </c>
       <c r="G57" s="24" t="inlineStr">
         <is>
-          <t>簽名映像正常；未簽名映像被拒；讀出的 flash 是密文</t>
-        </is>
-      </c>
-      <c r="H57" s="24" t="inlineStr">
-        <is>
-          <t>P0-14</t>
-        </is>
-      </c>
+          <t>100% 婉拒</t>
+        </is>
+      </c>
+      <c r="H57" s="24" t="inlineStr"/>
       <c r="I57" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -4398,47 +4410,39 @@
         <f>IF(J57="已完成",IF(K57="","",MAX(0,K57-F57)),IF(TODAY()&gt;F57,TODAY()-F57,""))</f>
         <v/>
       </c>
-      <c r="M57" s="24" t="inlineStr">
-        <is>
-          <t>燒 eFuse 不可逆，用一片專用測試板</t>
-        </is>
-      </c>
+      <c r="M57" s="24" t="inlineStr"/>
     </row>
     <row r="58" ht="34" customHeight="1">
       <c r="A58" s="23" t="n">
         <v>52</v>
       </c>
-      <c r="B58" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
+      <c r="B58" s="23" t="inlineStr">
+        <is>
+          <t>開發</t>
         </is>
       </c>
       <c r="C58" s="24" t="inlineStr">
         <is>
-          <t>韌體：分區表和加密</t>
+          <t>RAG 知識庫（快活）</t>
         </is>
       </c>
       <c r="D58" s="24" t="inlineStr">
         <is>
-          <t>加密後的板子走一次配網、對話、OTA</t>
+          <t>按馬會審核意見修改</t>
         </is>
       </c>
       <c r="E58" s="25" t="n">
-        <v>46338</v>
+        <v>46370</v>
       </c>
       <c r="F58" s="25" t="n">
-        <v>46339</v>
+        <v>46381</v>
       </c>
       <c r="G58" s="24" t="inlineStr">
         <is>
-          <t>功能和加密前一樣；記錄開機時間</t>
-        </is>
-      </c>
-      <c r="H58" s="24" t="inlineStr">
-        <is>
-          <t>P0-14</t>
-        </is>
-      </c>
+          <t>每次修改都有新版本和審批記錄</t>
+        </is>
+      </c>
+      <c r="H58" s="24" t="inlineStr"/>
       <c r="I58" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -4460,37 +4464,33 @@
       <c r="A59" s="23" t="n">
         <v>53</v>
       </c>
-      <c r="B59" s="23" t="inlineStr">
-        <is>
-          <t>開發</t>
+      <c r="B59" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
         </is>
       </c>
       <c r="C59" s="24" t="inlineStr">
         <is>
-          <t>韌體：分區表和加密</t>
+          <t>RAG 知識庫（快活）</t>
         </is>
       </c>
       <c r="D59" s="24" t="inlineStr">
         <is>
-          <t>分區表和加密設定凍結，寫進文件</t>
+          <t>在後台更新知識庫，用已出廠的玩具提問</t>
         </is>
       </c>
       <c r="E59" s="25" t="n">
-        <v>46339</v>
+        <v>46377</v>
       </c>
       <c r="F59" s="25" t="n">
-        <v>46339</v>
+        <v>46381</v>
       </c>
       <c r="G59" s="24" t="inlineStr">
         <is>
-          <t>之後不再改；文件寫明分區和 eFuse 設定</t>
-        </is>
-      </c>
-      <c r="H59" s="24" t="inlineStr">
-        <is>
-          <t>P2-12、P0-14</t>
-        </is>
-      </c>
+          <t>不用重新燒錄，玩具即時用新版本回答</t>
+        </is>
+      </c>
+      <c r="H59" s="24" t="inlineStr"/>
       <c r="I59" s="24" t="inlineStr">
         <is>
           <t>Jacky</t>
@@ -4506,11 +4506,7 @@
         <f>IF(J59="已完成",IF(K59="","",MAX(0,K59-F59)),IF(TODAY()&gt;F59,TODAY()-F59,""))</f>
         <v/>
       </c>
-      <c r="M59" s="24" t="inlineStr">
-        <is>
-          <t>11/13 凍結</t>
-        </is>
-      </c>
+      <c r="M59" s="24" t="inlineStr"/>
     </row>
     <row r="60" ht="34" customHeight="1">
       <c r="A60" s="20" t="n">
@@ -4523,28 +4519,28 @@
       </c>
       <c r="C60" s="21" t="inlineStr">
         <is>
-          <t>韌體：按品牌連線</t>
+          <t>韌體：分區表和加密</t>
         </is>
       </c>
       <c r="D60" s="21" t="inlineStr">
         <is>
-          <t>伺服器網址改從出廠設定讀取（品牌、網址）</t>
+          <t>新分區表：加大 app 分區，加品牌資源分區和出廠設定分區</t>
         </is>
       </c>
       <c r="E60" s="22" t="n">
-        <v>46328</v>
+        <v>46314</v>
       </c>
       <c r="F60" s="22" t="n">
-        <v>46336</v>
+        <v>46325</v>
       </c>
       <c r="G60" s="21" t="inlineStr">
         <is>
-          <t>程式碼裡不再寫死 elatoai.hkqft.com</t>
+          <t>新分區表能放下現在的韌體加 30% 空間</t>
         </is>
       </c>
       <c r="H60" s="21" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>P2-12</t>
         </is>
       </c>
       <c r="I60" s="21" t="inlineStr">
@@ -4568,35 +4564,35 @@
       <c r="A61" s="23" t="n">
         <v>55</v>
       </c>
-      <c r="B61" s="23" t="inlineStr">
-        <is>
-          <t>開發</t>
+      <c r="B61" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
         </is>
       </c>
       <c r="C61" s="24" t="inlineStr">
         <is>
-          <t>韌體：按品牌連線</t>
+          <t>韌體：分區表和加密</t>
         </is>
       </c>
       <c r="D61" s="24" t="inlineStr">
         <is>
-          <t>出廠設定是空白時不連任何正式伺服器，進入出廠模式</t>
+          <t>新分區表上做 OTA 升級和回滾各一次</t>
         </is>
       </c>
       <c r="E61" s="25" t="n">
-        <v>46335</v>
+        <v>46328</v>
       </c>
       <c r="F61" s="25" t="n">
-        <v>46337</v>
+        <v>46330</v>
       </c>
       <c r="G61" s="24" t="inlineStr">
         <is>
-          <t>空白板開機後停在出廠模式</t>
+          <t>兩次都成功</t>
         </is>
       </c>
       <c r="H61" s="24" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>P2-12、P0-13</t>
         </is>
       </c>
       <c r="I61" s="24" t="inlineStr">
@@ -4620,35 +4616,35 @@
       <c r="A62" s="23" t="n">
         <v>56</v>
       </c>
-      <c r="B62" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
+      <c r="B62" s="23" t="inlineStr">
+        <is>
+          <t>開發</t>
         </is>
       </c>
       <c r="C62" s="24" t="inlineStr">
         <is>
-          <t>韌體：按品牌連線</t>
+          <t>韌體：分區表和加密</t>
         </is>
       </c>
       <c r="D62" s="24" t="inlineStr">
         <is>
-          <t>兩片板寫入不同品牌，各自開機</t>
+          <t>產生 Secure Boot 簽名金鑰，離線備份兩份</t>
         </is>
       </c>
       <c r="E62" s="25" t="n">
-        <v>46338</v>
+        <v>46328</v>
       </c>
       <c r="F62" s="25" t="n">
-        <v>46339</v>
+        <v>46332</v>
       </c>
       <c r="G62" s="24" t="inlineStr">
         <is>
-          <t>各自連上自己那套系統；清空設定後不連任何正式伺服器</t>
+          <t>金鑰不在 repo、不在伺服器；備份放在兩個地方</t>
         </is>
       </c>
       <c r="H62" s="24" t="inlineStr">
         <is>
-          <t>R-35</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="I62" s="24" t="inlineStr">
@@ -4668,65 +4664,61 @@
       </c>
       <c r="M62" s="24" t="inlineStr">
         <is>
-          <t>需要第二套系統先臨時跑起來</t>
+          <t>金鑰遺失 = 所有玩具不能再 OTA</t>
         </is>
       </c>
     </row>
     <row r="63" ht="34" customHeight="1">
-      <c r="A63" s="20" t="n">
+      <c r="A63" s="23" t="n">
         <v>57</v>
       </c>
-      <c r="B63" s="20" t="inlineStr">
+      <c r="B63" s="23" t="inlineStr">
         <is>
           <t>開發</t>
         </is>
       </c>
-      <c r="C63" s="21" t="inlineStr">
-        <is>
-          <t>角色和內容</t>
-        </is>
-      </c>
-      <c r="D63" s="21" t="inlineStr">
-        <is>
-          <t>把 Navy 的人設、開場白、提示語、聲線放進系統（快活、政協青年聯會）</t>
-        </is>
-      </c>
-      <c r="E63" s="22" t="n">
-        <v>46335</v>
-      </c>
-      <c r="F63" s="22" t="n">
-        <v>46338</v>
-      </c>
-      <c r="G63" s="21" t="inlineStr">
-        <is>
-          <t>每個角色都能選、能對話</t>
-        </is>
-      </c>
-      <c r="H63" s="21" t="inlineStr">
-        <is>
-          <t>R-24</t>
-        </is>
-      </c>
-      <c r="I63" s="21" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J63" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K63" s="22" t="n"/>
-      <c r="L63" s="20">
+      <c r="C63" s="24" t="inlineStr">
+        <is>
+          <t>韌體：分區表和加密</t>
+        </is>
+      </c>
+      <c r="D63" s="24" t="inlineStr">
+        <is>
+          <t>編譯流程加簽名和 Flash 加密</t>
+        </is>
+      </c>
+      <c r="E63" s="25" t="n">
+        <v>46330</v>
+      </c>
+      <c r="F63" s="25" t="n">
+        <v>46336</v>
+      </c>
+      <c r="G63" s="24" t="inlineStr">
+        <is>
+          <t>一條命令出簽名後的正式映像</t>
+        </is>
+      </c>
+      <c r="H63" s="24" t="inlineStr">
+        <is>
+          <t>P0-14</t>
+        </is>
+      </c>
+      <c r="I63" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J63" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K63" s="25" t="n"/>
+      <c r="L63" s="23">
         <f>IF(J63="已完成",IF(K63="","",MAX(0,K63-F63)),IF(TODAY()&gt;F63,TODAY()-F63,""))</f>
         <v/>
       </c>
-      <c r="M63" s="21" t="inlineStr">
-        <is>
-          <t>Navy 11/13 定稿，初稿先放</t>
-        </is>
-      </c>
+      <c r="M63" s="24" t="inlineStr"/>
     </row>
     <row r="64" ht="34" customHeight="1">
       <c r="A64" s="23" t="n">
@@ -4739,33 +4731,33 @@
       </c>
       <c r="C64" s="24" t="inlineStr">
         <is>
-          <t>角色和內容</t>
+          <t>韌體：分區表和加密</t>
         </is>
       </c>
       <c r="D64" s="24" t="inlineStr">
         <is>
-          <t>每個角色試聽 20 句，錄音給客戶確認</t>
+          <t>一片測試板燒 eFuse：簽名映像開機、未簽名映像 OTA、讀出 flash</t>
         </is>
       </c>
       <c r="E64" s="25" t="n">
-        <v>46338</v>
+        <v>46337</v>
       </c>
       <c r="F64" s="25" t="n">
         <v>46339</v>
       </c>
       <c r="G64" s="24" t="inlineStr">
         <is>
-          <t>客戶確認每個角色</t>
+          <t>簽名映像正常；未簽名映像被拒；讀出的 flash 是密文</t>
         </is>
       </c>
       <c r="H64" s="24" t="inlineStr">
         <is>
-          <t>R-24</t>
+          <t>P0-14</t>
         </is>
       </c>
       <c r="I64" s="24" t="inlineStr">
         <is>
-          <t>Jacky、Navy</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="J64" s="23" t="inlineStr">
@@ -4778,63 +4770,63 @@
         <f>IF(J64="已完成",IF(K64="","",MAX(0,K64-F64)),IF(TODAY()&gt;F64,TODAY()-F64,""))</f>
         <v/>
       </c>
-      <c r="M64" s="24" t="inlineStr"/>
+      <c r="M64" s="24" t="inlineStr">
+        <is>
+          <t>燒 eFuse 不可逆，用一片專用測試板</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="34" customHeight="1">
-      <c r="A65" s="20" t="n">
+      <c r="A65" s="23" t="n">
         <v>59</v>
       </c>
-      <c r="B65" s="20" t="inlineStr">
-        <is>
-          <t>開發</t>
-        </is>
-      </c>
-      <c r="C65" s="21" t="inlineStr">
-        <is>
-          <t>網頁：功能開關和政協</t>
-        </is>
-      </c>
-      <c r="D65" s="21" t="inlineStr">
-        <is>
-          <t>會員綁定</t>
-        </is>
-      </c>
-      <c r="E65" s="22" t="n">
-        <v>46335</v>
-      </c>
-      <c r="F65" s="22" t="n">
-        <v>46342</v>
-      </c>
-      <c r="G65" s="21" t="inlineStr">
-        <is>
-          <t>按 Q12 的決定完成（我們自己的帳號或馬會登入）</t>
-        </is>
-      </c>
-      <c r="H65" s="21" t="inlineStr">
-        <is>
-          <t>R-30、Q12</t>
-        </is>
-      </c>
-      <c r="I65" s="21" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J65" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K65" s="22" t="n"/>
-      <c r="L65" s="20">
+      <c r="B65" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="C65" s="24" t="inlineStr">
+        <is>
+          <t>韌體：分區表和加密</t>
+        </is>
+      </c>
+      <c r="D65" s="24" t="inlineStr">
+        <is>
+          <t>加密後的板子走一次配網、對話、OTA</t>
+        </is>
+      </c>
+      <c r="E65" s="25" t="n">
+        <v>46338</v>
+      </c>
+      <c r="F65" s="25" t="n">
+        <v>46339</v>
+      </c>
+      <c r="G65" s="24" t="inlineStr">
+        <is>
+          <t>功能和加密前一樣；記錄開機時間</t>
+        </is>
+      </c>
+      <c r="H65" s="24" t="inlineStr">
+        <is>
+          <t>P0-14</t>
+        </is>
+      </c>
+      <c r="I65" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J65" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K65" s="25" t="n"/>
+      <c r="L65" s="23">
         <f>IF(J65="已完成",IF(K65="","",MAX(0,K65-F65)),IF(TODAY()&gt;F65,TODAY()-F65,""))</f>
         <v/>
       </c>
-      <c r="M65" s="21" t="inlineStr">
-        <is>
-          <t>要先回答 Q12</t>
-        </is>
-      </c>
+      <c r="M65" s="24" t="inlineStr"/>
     </row>
     <row r="66" ht="34" customHeight="1">
       <c r="A66" s="23" t="n">
@@ -4847,28 +4839,28 @@
       </c>
       <c r="C66" s="24" t="inlineStr">
         <is>
-          <t>網頁：功能開關和政協</t>
+          <t>韌體：分區表和加密</t>
         </is>
       </c>
       <c r="D66" s="24" t="inlineStr">
         <is>
-          <t>查看記憶、一鍵忘記</t>
+          <t>分區表和加密設定凍結，寫進文件</t>
         </is>
       </c>
       <c r="E66" s="25" t="n">
-        <v>46335</v>
+        <v>46339</v>
       </c>
       <c r="F66" s="25" t="n">
         <v>46339</v>
       </c>
       <c r="G66" s="24" t="inlineStr">
         <is>
-          <t>看到的記憶只屬於自己的設備；忘記後不會再出現</t>
+          <t>之後不再改；文件寫明分區和 eFuse 設定</t>
         </is>
       </c>
       <c r="H66" s="24" t="inlineStr">
         <is>
-          <t>R-30、P1-12</t>
+          <t>P2-12、P0-14</t>
         </is>
       </c>
       <c r="I66" s="24" t="inlineStr">
@@ -4886,59 +4878,63 @@
         <f>IF(J66="已完成",IF(K66="","",MAX(0,K66-F66)),IF(TODAY()&gt;F66,TODAY()-F66,""))</f>
         <v/>
       </c>
-      <c r="M66" s="24" t="inlineStr"/>
+      <c r="M66" s="24" t="inlineStr">
+        <is>
+          <t>11/13 凍結</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="34" customHeight="1">
-      <c r="A67" s="23" t="n">
+      <c r="A67" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="B67" s="23" t="inlineStr">
+      <c r="B67" s="20" t="inlineStr">
         <is>
           <t>開發</t>
         </is>
       </c>
-      <c r="C67" s="24" t="inlineStr">
-        <is>
-          <t>網頁：功能開關和政協</t>
-        </is>
-      </c>
-      <c r="D67" s="24" t="inlineStr">
-        <is>
-          <t>選語言（粵、普、英）：介面和語音回答都跟著切換</t>
-        </is>
-      </c>
-      <c r="E67" s="25" t="n">
-        <v>46339</v>
-      </c>
-      <c r="F67" s="25" t="n">
-        <v>46344</v>
-      </c>
-      <c r="G67" s="24" t="inlineStr">
-        <is>
-          <t>三種語言的介面和回答都正確</t>
-        </is>
-      </c>
-      <c r="H67" s="24" t="inlineStr">
-        <is>
-          <t>R-30</t>
-        </is>
-      </c>
-      <c r="I67" s="24" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J67" s="23" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K67" s="25" t="n"/>
-      <c r="L67" s="23">
+      <c r="C67" s="21" t="inlineStr">
+        <is>
+          <t>韌體：按品牌連線</t>
+        </is>
+      </c>
+      <c r="D67" s="21" t="inlineStr">
+        <is>
+          <t>伺服器網址改從出廠設定讀取（品牌、網址）</t>
+        </is>
+      </c>
+      <c r="E67" s="22" t="n">
+        <v>46328</v>
+      </c>
+      <c r="F67" s="22" t="n">
+        <v>46336</v>
+      </c>
+      <c r="G67" s="21" t="inlineStr">
+        <is>
+          <t>程式碼裡不再寫死 elatoai.hkqft.com</t>
+        </is>
+      </c>
+      <c r="H67" s="21" t="inlineStr">
+        <is>
+          <t>R-35</t>
+        </is>
+      </c>
+      <c r="I67" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J67" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K67" s="22" t="n"/>
+      <c r="L67" s="20">
         <f>IF(J67="已完成",IF(K67="","",MAX(0,K67-F67)),IF(TODAY()&gt;F67,TODAY()-F67,""))</f>
         <v/>
       </c>
-      <c r="M67" s="24" t="inlineStr"/>
+      <c r="M67" s="21" t="inlineStr"/>
     </row>
     <row r="68" ht="34" customHeight="1">
       <c r="A68" s="23" t="n">
@@ -4951,28 +4947,28 @@
       </c>
       <c r="C68" s="24" t="inlineStr">
         <is>
-          <t>網頁：功能開關和政協</t>
+          <t>韌體：按品牌連線</t>
         </is>
       </c>
       <c r="D68" s="24" t="inlineStr">
         <is>
-          <t>政協青年聯會的外觀包和角色，用成人版流程</t>
+          <t>出廠設定是空白時不連任何正式伺服器，進入出廠模式</t>
         </is>
       </c>
       <c r="E68" s="25" t="n">
-        <v>46342</v>
+        <v>46335</v>
       </c>
       <c r="F68" s="25" t="n">
-        <v>46345</v>
+        <v>46337</v>
       </c>
       <c r="G68" s="24" t="inlineStr">
         <is>
-          <t>只換外觀和角色，沒有另寫頁面</t>
+          <t>空白板開機後停在出廠模式</t>
         </is>
       </c>
       <c r="H68" s="24" t="inlineStr">
         <is>
-          <t>R-31</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="I68" s="24" t="inlineStr">
@@ -5003,28 +4999,28 @@
       </c>
       <c r="C69" s="24" t="inlineStr">
         <is>
-          <t>網頁：功能開關和政協</t>
+          <t>韌體：按品牌連線</t>
         </is>
       </c>
       <c r="D69" s="24" t="inlineStr">
         <is>
-          <t>快活每個功能開關打開、關閉各測一次</t>
+          <t>兩片板寫入不同品牌，各自開機</t>
         </is>
       </c>
       <c r="E69" s="25" t="n">
-        <v>46346</v>
+        <v>46338</v>
       </c>
       <c r="F69" s="25" t="n">
-        <v>46346</v>
+        <v>46339</v>
       </c>
       <c r="G69" s="24" t="inlineStr">
         <is>
-          <t>關閉時入口不出現；打開時功能正常</t>
+          <t>各自連上自己那套系統；清空設定後不連任何正式伺服器</t>
         </is>
       </c>
       <c r="H69" s="24" t="inlineStr">
         <is>
-          <t>R-30</t>
+          <t>R-35</t>
         </is>
       </c>
       <c r="I69" s="24" t="inlineStr">
@@ -5042,163 +5038,175 @@
         <f>IF(J69="已完成",IF(K69="","",MAX(0,K69-F69)),IF(TODAY()&gt;F69,TODAY()-F69,""))</f>
         <v/>
       </c>
-      <c r="M69" s="24" t="inlineStr"/>
+      <c r="M69" s="24" t="inlineStr">
+        <is>
+          <t>需要第二套系統先臨時跑起來</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="34" customHeight="1">
-      <c r="A70" s="23" t="n">
+      <c r="A70" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="B70" s="26" t="inlineStr">
+      <c r="B70" s="20" t="inlineStr">
+        <is>
+          <t>開發</t>
+        </is>
+      </c>
+      <c r="C70" s="21" t="inlineStr">
+        <is>
+          <t>角色和內容</t>
+        </is>
+      </c>
+      <c r="D70" s="21" t="inlineStr">
+        <is>
+          <t>把 Navy 的人設、開場白、提示語、聲線放進系統（快活、政協青年聯會）</t>
+        </is>
+      </c>
+      <c r="E70" s="22" t="n">
+        <v>46335</v>
+      </c>
+      <c r="F70" s="22" t="n">
+        <v>46338</v>
+      </c>
+      <c r="G70" s="21" t="inlineStr">
+        <is>
+          <t>每個角色都能選、能對話</t>
+        </is>
+      </c>
+      <c r="H70" s="21" t="inlineStr">
+        <is>
+          <t>R-24</t>
+        </is>
+      </c>
+      <c r="I70" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J70" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K70" s="22" t="n"/>
+      <c r="L70" s="20">
+        <f>IF(J70="已完成",IF(K70="","",MAX(0,K70-F70)),IF(TODAY()&gt;F70,TODAY()-F70,""))</f>
+        <v/>
+      </c>
+      <c r="M70" s="21" t="inlineStr">
+        <is>
+          <t>Navy 11/13 定稿，初稿先放</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="34" customHeight="1">
+      <c r="A71" s="23" t="n">
+        <v>65</v>
+      </c>
+      <c r="B71" s="26" t="inlineStr">
         <is>
           <t>測試</t>
         </is>
       </c>
-      <c r="C70" s="24" t="inlineStr">
+      <c r="C71" s="24" t="inlineStr">
+        <is>
+          <t>角色和內容</t>
+        </is>
+      </c>
+      <c r="D71" s="24" t="inlineStr">
+        <is>
+          <t>每個角色試聽 20 句，錄音給客戶確認</t>
+        </is>
+      </c>
+      <c r="E71" s="25" t="n">
+        <v>46338</v>
+      </c>
+      <c r="F71" s="25" t="n">
+        <v>46339</v>
+      </c>
+      <c r="G71" s="24" t="inlineStr">
+        <is>
+          <t>客戶確認每個角色</t>
+        </is>
+      </c>
+      <c r="H71" s="24" t="inlineStr">
+        <is>
+          <t>R-24</t>
+        </is>
+      </c>
+      <c r="I71" s="24" t="inlineStr">
+        <is>
+          <t>Jacky、Navy</t>
+        </is>
+      </c>
+      <c r="J71" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K71" s="25" t="n"/>
+      <c r="L71" s="23">
+        <f>IF(J71="已完成",IF(K71="","",MAX(0,K71-F71)),IF(TODAY()&gt;F71,TODAY()-F71,""))</f>
+        <v/>
+      </c>
+      <c r="M71" s="24" t="inlineStr"/>
+    </row>
+    <row r="72" ht="34" customHeight="1">
+      <c r="A72" s="20" t="n">
+        <v>66</v>
+      </c>
+      <c r="B72" s="20" t="inlineStr">
+        <is>
+          <t>開發</t>
+        </is>
+      </c>
+      <c r="C72" s="21" t="inlineStr">
         <is>
           <t>網頁：功能開關和政協</t>
         </is>
       </c>
-      <c r="D70" s="24" t="inlineStr">
-        <is>
-          <t>政協青年聯會版走一次全流程</t>
-        </is>
-      </c>
-      <c r="E70" s="25" t="n">
-        <v>46346</v>
-      </c>
-      <c r="F70" s="25" t="n">
-        <v>46346</v>
-      </c>
-      <c r="G70" s="24" t="inlineStr">
-        <is>
-          <t>全部正常；介面沒有出現「快活」或馬會字樣</t>
-        </is>
-      </c>
-      <c r="H70" s="24" t="inlineStr">
-        <is>
-          <t>R-31</t>
-        </is>
-      </c>
-      <c r="I70" s="24" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J70" s="23" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K70" s="25" t="n"/>
-      <c r="L70" s="23">
-        <f>IF(J70="已完成",IF(K70="","",MAX(0,K70-F70)),IF(TODAY()&gt;F70,TODAY()-F70,""))</f>
-        <v/>
-      </c>
-      <c r="M70" s="24" t="inlineStr"/>
-    </row>
-    <row r="71" ht="34" customHeight="1">
-      <c r="A71" s="20" t="n">
-        <v>65</v>
-      </c>
-      <c r="B71" s="20" t="inlineStr">
-        <is>
-          <t>開發</t>
-        </is>
-      </c>
-      <c r="C71" s="21" t="inlineStr">
-        <is>
-          <t>後台管理</t>
-        </is>
-      </c>
-      <c r="D71" s="21" t="inlineStr">
-        <is>
-          <t>內容管理員：上載知識庫並送審、發佈角色</t>
-        </is>
-      </c>
-      <c r="E71" s="22" t="n">
-        <v>46328</v>
-      </c>
-      <c r="F71" s="22" t="n">
-        <v>46339</v>
-      </c>
-      <c r="G71" s="21" t="inlineStr">
-        <is>
-          <t>可以上載、送審、發佈</t>
-        </is>
-      </c>
-      <c r="H71" s="21" t="inlineStr">
-        <is>
-          <t>P0-12</t>
-        </is>
-      </c>
-      <c r="I71" s="21" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J71" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K71" s="22" t="n"/>
-      <c r="L71" s="20">
-        <f>IF(J71="已完成",IF(K71="","",MAX(0,K71-F71)),IF(TODAY()&gt;F71,TODAY()-F71,""))</f>
-        <v/>
-      </c>
-      <c r="M71" s="21" t="inlineStr"/>
-    </row>
-    <row r="72" ht="34" customHeight="1">
-      <c r="A72" s="23" t="n">
-        <v>66</v>
-      </c>
-      <c r="B72" s="23" t="inlineStr">
-        <is>
-          <t>開發</t>
-        </is>
-      </c>
-      <c r="C72" s="24" t="inlineStr">
-        <is>
-          <t>後台管理</t>
-        </is>
-      </c>
-      <c r="D72" s="24" t="inlineStr">
-        <is>
-          <t>超級管理員：設備列表（最後上線、韌體版本、錯誤）</t>
-        </is>
-      </c>
-      <c r="E72" s="25" t="n">
+      <c r="D72" s="21" t="inlineStr">
+        <is>
+          <t>會員綁定</t>
+        </is>
+      </c>
+      <c r="E72" s="22" t="n">
         <v>46335</v>
       </c>
-      <c r="F72" s="25" t="n">
-        <v>46343</v>
-      </c>
-      <c r="G72" s="24" t="inlineStr">
-        <is>
-          <t>每台設備的狀態一目了然</t>
-        </is>
-      </c>
-      <c r="H72" s="24" t="inlineStr">
-        <is>
-          <t>R-11</t>
-        </is>
-      </c>
-      <c r="I72" s="24" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J72" s="23" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K72" s="25" t="n"/>
-      <c r="L72" s="23">
+      <c r="F72" s="22" t="n">
+        <v>46342</v>
+      </c>
+      <c r="G72" s="21" t="inlineStr">
+        <is>
+          <t>按 Q12 的決定完成（我們自己的帳號或馬會登入）</t>
+        </is>
+      </c>
+      <c r="H72" s="21" t="inlineStr">
+        <is>
+          <t>R-30、Q12</t>
+        </is>
+      </c>
+      <c r="I72" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J72" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K72" s="22" t="n"/>
+      <c r="L72" s="20">
         <f>IF(J72="已完成",IF(K72="","",MAX(0,K72-F72)),IF(TODAY()&gt;F72,TODAY()-F72,""))</f>
         <v/>
       </c>
-      <c r="M72" s="24" t="inlineStr"/>
+      <c r="M72" s="21" t="inlineStr">
+        <is>
+          <t>要先回答 Q12</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="34" customHeight="1">
       <c r="A73" s="23" t="n">
@@ -5211,28 +5219,28 @@
       </c>
       <c r="C73" s="24" t="inlineStr">
         <is>
-          <t>後台管理</t>
+          <t>網頁：功能開關和政協</t>
         </is>
       </c>
       <c r="D73" s="24" t="inlineStr">
         <is>
-          <t>超級管理員：發佈 OTA、解綁、換機</t>
+          <t>查看記憶、一鍵忘記</t>
         </is>
       </c>
       <c r="E73" s="25" t="n">
+        <v>46335</v>
+      </c>
+      <c r="F73" s="25" t="n">
         <v>46339</v>
       </c>
-      <c r="F73" s="25" t="n">
-        <v>46345</v>
-      </c>
       <c r="G73" s="24" t="inlineStr">
         <is>
-          <t>三項操作都可以在後台完成</t>
+          <t>看到的記憶只屬於自己的設備；忘記後不會再出現</t>
         </is>
       </c>
       <c r="H73" s="24" t="inlineStr">
         <is>
-          <t>R-11、P0-13</t>
+          <t>R-30、P1-12</t>
         </is>
       </c>
       <c r="I73" s="24" t="inlineStr">
@@ -5252,39 +5260,39 @@
       </c>
       <c r="M73" s="24" t="inlineStr"/>
     </row>
-    <row r="74" ht="49" customHeight="1">
+    <row r="74" ht="34" customHeight="1">
       <c r="A74" s="23" t="n">
         <v>68</v>
       </c>
-      <c r="B74" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
+      <c r="B74" s="23" t="inlineStr">
+        <is>
+          <t>開發</t>
         </is>
       </c>
       <c r="C74" s="24" t="inlineStr">
         <is>
-          <t>後台管理</t>
+          <t>網頁：功能開關和政協</t>
         </is>
       </c>
       <c r="D74" s="24" t="inlineStr">
         <is>
-          <t>權限測試：內容管理員、超級管理員、普通用戶各登入一次</t>
+          <t>選語言（粵、普、英）：介面和語音回答都跟著切換</t>
         </is>
       </c>
       <c r="E74" s="25" t="n">
-        <v>46346</v>
+        <v>46339</v>
       </c>
       <c r="F74" s="25" t="n">
-        <v>46346</v>
+        <v>46344</v>
       </c>
       <c r="G74" s="24" t="inlineStr">
         <is>
-          <t>每種角色只看到自己可以做的；任何管理員都看不到對話內容（網頁和資料庫兩層都查）</t>
+          <t>三種語言的介面和回答都正確</t>
         </is>
       </c>
       <c r="H74" s="24" t="inlineStr">
         <is>
-          <t>P0-12</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="I74" s="24" t="inlineStr">
@@ -5305,58 +5313,58 @@
       <c r="M74" s="24" t="inlineStr"/>
     </row>
     <row r="75" ht="34" customHeight="1">
-      <c r="A75" s="20" t="n">
+      <c r="A75" s="23" t="n">
         <v>69</v>
       </c>
-      <c r="B75" s="20" t="inlineStr">
+      <c r="B75" s="23" t="inlineStr">
         <is>
           <t>開發</t>
         </is>
       </c>
-      <c r="C75" s="21" t="inlineStr">
-        <is>
-          <t>內部測試</t>
-        </is>
-      </c>
-      <c r="D75" s="21" t="inlineStr">
-        <is>
-          <t>每週數據報表：對話輪數、首字延遲、每台成本、安全事件</t>
-        </is>
-      </c>
-      <c r="E75" s="22" t="n">
-        <v>46328</v>
-      </c>
-      <c r="F75" s="22" t="n">
-        <v>46332</v>
-      </c>
-      <c r="G75" s="21" t="inlineStr">
-        <is>
-          <t>一條命令出報表</t>
-        </is>
-      </c>
-      <c r="H75" s="21" t="inlineStr">
-        <is>
-          <t>R-07、P2-09</t>
-        </is>
-      </c>
-      <c r="I75" s="21" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J75" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K75" s="22" t="n"/>
-      <c r="L75" s="20">
+      <c r="C75" s="24" t="inlineStr">
+        <is>
+          <t>網頁：功能開關和政協</t>
+        </is>
+      </c>
+      <c r="D75" s="24" t="inlineStr">
+        <is>
+          <t>政協青年聯會的外觀包和角色，用成人版流程</t>
+        </is>
+      </c>
+      <c r="E75" s="25" t="n">
+        <v>46342</v>
+      </c>
+      <c r="F75" s="25" t="n">
+        <v>46345</v>
+      </c>
+      <c r="G75" s="24" t="inlineStr">
+        <is>
+          <t>只換外觀和角色，沒有另寫頁面</t>
+        </is>
+      </c>
+      <c r="H75" s="24" t="inlineStr">
+        <is>
+          <t>R-31</t>
+        </is>
+      </c>
+      <c r="I75" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J75" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K75" s="25" t="n"/>
+      <c r="L75" s="23">
         <f>IF(J75="已完成",IF(K75="","",MAX(0,K75-F75)),IF(TODAY()&gt;F75,TODAY()-F75,""))</f>
         <v/>
       </c>
-      <c r="M75" s="21" t="inlineStr"/>
-    </row>
-    <row r="76" ht="19" customHeight="1">
+      <c r="M75" s="24" t="inlineStr"/>
+    </row>
+    <row r="76" ht="34" customHeight="1">
       <c r="A76" s="23" t="n">
         <v>70</v>
       </c>
@@ -5367,33 +5375,33 @@
       </c>
       <c r="C76" s="24" t="inlineStr">
         <is>
-          <t>內部測試</t>
+          <t>網頁：功能開關和政協</t>
         </is>
       </c>
       <c r="D76" s="24" t="inlineStr">
         <is>
-          <t>20 台內部測試，每週出一次報表</t>
+          <t>快活每個功能開關打開、關閉各測一次</t>
         </is>
       </c>
       <c r="E76" s="25" t="n">
-        <v>46328</v>
+        <v>46346</v>
       </c>
       <c r="F76" s="25" t="n">
-        <v>46353</v>
+        <v>46346</v>
       </c>
       <c r="G76" s="24" t="inlineStr">
         <is>
-          <t>4 份週報齊全；第 4 週出測試報告</t>
+          <t>關閉時入口不出現；打開時功能正常</t>
         </is>
       </c>
       <c r="H76" s="24" t="inlineStr">
         <is>
-          <t>R-07</t>
+          <t>R-30</t>
         </is>
       </c>
       <c r="I76" s="24" t="inlineStr">
         <is>
-          <t>全體</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="J76" s="23" t="inlineStr">
@@ -5409,108 +5417,108 @@
       <c r="M76" s="24" t="inlineStr"/>
     </row>
     <row r="77" ht="34" customHeight="1">
-      <c r="A77" s="20" t="n">
+      <c r="A77" s="23" t="n">
         <v>71</v>
       </c>
-      <c r="B77" s="20" t="inlineStr">
+      <c r="B77" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="C77" s="24" t="inlineStr">
+        <is>
+          <t>網頁：功能開關和政協</t>
+        </is>
+      </c>
+      <c r="D77" s="24" t="inlineStr">
+        <is>
+          <t>政協青年聯會版走一次全流程</t>
+        </is>
+      </c>
+      <c r="E77" s="25" t="n">
+        <v>46346</v>
+      </c>
+      <c r="F77" s="25" t="n">
+        <v>46346</v>
+      </c>
+      <c r="G77" s="24" t="inlineStr">
+        <is>
+          <t>全部正常；介面沒有出現「快活」或馬會字樣</t>
+        </is>
+      </c>
+      <c r="H77" s="24" t="inlineStr">
+        <is>
+          <t>R-31</t>
+        </is>
+      </c>
+      <c r="I77" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J77" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K77" s="25" t="n"/>
+      <c r="L77" s="23">
+        <f>IF(J77="已完成",IF(K77="","",MAX(0,K77-F77)),IF(TODAY()&gt;F77,TODAY()-F77,""))</f>
+        <v/>
+      </c>
+      <c r="M77" s="24" t="inlineStr"/>
+    </row>
+    <row r="78" ht="34" customHeight="1">
+      <c r="A78" s="20" t="n">
+        <v>72</v>
+      </c>
+      <c r="B78" s="20" t="inlineStr">
         <is>
           <t>開發</t>
         </is>
       </c>
-      <c r="C77" s="21" t="inlineStr">
-        <is>
-          <t>出廠模式和工位</t>
-        </is>
-      </c>
-      <c r="D77" s="21" t="inlineStr">
-        <is>
-          <t>韌體出廠模式：經序列埠寫入密鑰、品牌、款式</t>
-        </is>
-      </c>
-      <c r="E77" s="22" t="n">
-        <v>46342</v>
-      </c>
-      <c r="F77" s="22" t="n">
-        <v>46346</v>
-      </c>
-      <c r="G77" s="21" t="inlineStr">
-        <is>
-          <t>寫入後重新開機，連上該品牌系統</t>
-        </is>
-      </c>
-      <c r="H77" s="21" t="inlineStr">
-        <is>
-          <t>R-10</t>
-        </is>
-      </c>
-      <c r="I77" s="21" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J77" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K77" s="22" t="n"/>
-      <c r="L77" s="20">
-        <f>IF(J77="已完成",IF(K77="","",MAX(0,K77-F77)),IF(TODAY()&gt;F77,TODAY()-F77,""))</f>
-        <v/>
-      </c>
-      <c r="M77" s="21" t="inlineStr"/>
-    </row>
-    <row r="78" ht="34" customHeight="1">
-      <c r="A78" s="23" t="n">
-        <v>72</v>
-      </c>
-      <c r="B78" s="23" t="inlineStr">
-        <is>
-          <t>開發</t>
-        </is>
-      </c>
-      <c r="C78" s="24" t="inlineStr">
-        <is>
-          <t>出廠模式和工位</t>
-        </is>
-      </c>
-      <c r="D78" s="24" t="inlineStr">
-        <is>
-          <t>韌體自檢指令：喇叭、麥克風、按鍵、燈、Wi-Fi、電池</t>
-        </is>
-      </c>
-      <c r="E78" s="25" t="n">
-        <v>46342</v>
-      </c>
-      <c r="F78" s="25" t="n">
-        <v>46346</v>
-      </c>
-      <c r="G78" s="24" t="inlineStr">
-        <is>
-          <t>每項回傳通過或失敗</t>
-        </is>
-      </c>
-      <c r="H78" s="24" t="inlineStr">
-        <is>
-          <t>R-10</t>
-        </is>
-      </c>
-      <c r="I78" s="24" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J78" s="23" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K78" s="25" t="n"/>
-      <c r="L78" s="23">
+      <c r="C78" s="21" t="inlineStr">
+        <is>
+          <t>後台管理</t>
+        </is>
+      </c>
+      <c r="D78" s="21" t="inlineStr">
+        <is>
+          <t>內容管理員：上載知識庫並送審、發佈角色</t>
+        </is>
+      </c>
+      <c r="E78" s="22" t="n">
+        <v>46328</v>
+      </c>
+      <c r="F78" s="22" t="n">
+        <v>46339</v>
+      </c>
+      <c r="G78" s="21" t="inlineStr">
+        <is>
+          <t>可以上載、送審、發佈</t>
+        </is>
+      </c>
+      <c r="H78" s="21" t="inlineStr">
+        <is>
+          <t>P0-12</t>
+        </is>
+      </c>
+      <c r="I78" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J78" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K78" s="22" t="n"/>
+      <c r="L78" s="20">
         <f>IF(J78="已完成",IF(K78="","",MAX(0,K78-F78)),IF(TODAY()&gt;F78,TODAY()-F78,""))</f>
         <v/>
       </c>
-      <c r="M78" s="24" t="inlineStr"/>
+      <c r="M78" s="21" t="inlineStr"/>
     </row>
     <row r="79" ht="34" customHeight="1">
       <c r="A79" s="23" t="n">
@@ -5523,28 +5531,28 @@
       </c>
       <c r="C79" s="24" t="inlineStr">
         <is>
-          <t>出廠模式和工位</t>
+          <t>後台管理</t>
         </is>
       </c>
       <c r="D79" s="24" t="inlineStr">
         <is>
-          <t>工位腳本：讀 MAC、產生密鑰、寫入、自檢、登記、顯示結果</t>
+          <t>超級管理員：設備列表（最後上線、韌體版本、錯誤）</t>
         </is>
       </c>
       <c r="E79" s="25" t="n">
-        <v>46344</v>
+        <v>46335</v>
       </c>
       <c r="F79" s="25" t="n">
-        <v>46350</v>
+        <v>46343</v>
       </c>
       <c r="G79" s="24" t="inlineStr">
         <is>
-          <t>一條命令完成一台；結果用大字顯示通過或失敗</t>
+          <t>每台設備的狀態一目了然</t>
         </is>
       </c>
       <c r="H79" s="24" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-11</t>
         </is>
       </c>
       <c r="I79" s="24" t="inlineStr">
@@ -5575,28 +5583,28 @@
       </c>
       <c r="C80" s="24" t="inlineStr">
         <is>
-          <t>出廠模式和工位</t>
+          <t>後台管理</t>
         </is>
       </c>
       <c r="D80" s="24" t="inlineStr">
         <is>
-          <t>每套系統加登記接口（工位專用憑證）</t>
+          <t>超級管理員：發佈 OTA、解綁、換機</t>
         </is>
       </c>
       <c r="E80" s="25" t="n">
-        <v>46346</v>
+        <v>46339</v>
       </c>
       <c r="F80" s="25" t="n">
-        <v>46350</v>
+        <v>46345</v>
       </c>
       <c r="G80" s="24" t="inlineStr">
         <is>
-          <t>只有工位能登記；同一台不能重複登記</t>
+          <t>三項操作都可以在後台完成</t>
         </is>
       </c>
       <c r="H80" s="24" t="inlineStr">
         <is>
-          <t>R-10、R-34</t>
+          <t>R-11、P0-13</t>
         </is>
       </c>
       <c r="I80" s="24" t="inlineStr">
@@ -5616,7 +5624,7 @@
       </c>
       <c r="M80" s="24" t="inlineStr"/>
     </row>
-    <row r="81" ht="34" customHeight="1">
+    <row r="81" ht="49" customHeight="1">
       <c r="A81" s="23" t="n">
         <v>75</v>
       </c>
@@ -5627,28 +5635,28 @@
       </c>
       <c r="C81" s="24" t="inlineStr">
         <is>
-          <t>出廠模式和工位</t>
+          <t>後台管理</t>
         </is>
       </c>
       <c r="D81" s="24" t="inlineStr">
         <is>
-          <t>連續 10 台過工位</t>
+          <t>權限測試：內容管理員、超級管理員、普通用戶各登入一次</t>
         </is>
       </c>
       <c r="E81" s="25" t="n">
-        <v>46351</v>
+        <v>46346</v>
       </c>
       <c r="F81" s="25" t="n">
-        <v>46353</v>
+        <v>46346</v>
       </c>
       <c r="G81" s="24" t="inlineStr">
         <is>
-          <t>10 台全部通過；每台不超過 1.5 分鐘</t>
+          <t>每種角色只看到自己可以做的；任何管理員都看不到對話內容（網頁和資料庫兩層都查）</t>
         </is>
       </c>
       <c r="H81" s="24" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>P0-12</t>
         </is>
       </c>
       <c r="I81" s="24" t="inlineStr">
@@ -5669,95 +5677,95 @@
       <c r="M81" s="24" t="inlineStr"/>
     </row>
     <row r="82" ht="34" customHeight="1">
-      <c r="A82" s="23" t="n">
+      <c r="A82" s="20" t="n">
         <v>76</v>
       </c>
-      <c r="B82" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
-        </is>
-      </c>
-      <c r="C82" s="24" t="inlineStr">
-        <is>
-          <t>出廠模式和工位</t>
-        </is>
-      </c>
-      <c r="D82" s="24" t="inlineStr">
-        <is>
-          <t>混入壞板：拔掉喇叭、拔掉麥克風、低電、重複登記</t>
-        </is>
-      </c>
-      <c r="E82" s="25" t="n">
-        <v>46351</v>
-      </c>
-      <c r="F82" s="25" t="n">
-        <v>46353</v>
-      </c>
-      <c r="G82" s="24" t="inlineStr">
-        <is>
-          <t>每種都被攔下並顯示原因</t>
-        </is>
-      </c>
-      <c r="H82" s="24" t="inlineStr">
-        <is>
-          <t>R-10</t>
-        </is>
-      </c>
-      <c r="I82" s="24" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J82" s="23" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K82" s="25" t="n"/>
-      <c r="L82" s="23">
+      <c r="B82" s="20" t="inlineStr">
+        <is>
+          <t>開發</t>
+        </is>
+      </c>
+      <c r="C82" s="21" t="inlineStr">
+        <is>
+          <t>內部測試</t>
+        </is>
+      </c>
+      <c r="D82" s="21" t="inlineStr">
+        <is>
+          <t>每週數據報表：對話輪數、首字延遲、每台成本、安全事件</t>
+        </is>
+      </c>
+      <c r="E82" s="22" t="n">
+        <v>46328</v>
+      </c>
+      <c r="F82" s="22" t="n">
+        <v>46332</v>
+      </c>
+      <c r="G82" s="21" t="inlineStr">
+        <is>
+          <t>一條命令出報表</t>
+        </is>
+      </c>
+      <c r="H82" s="21" t="inlineStr">
+        <is>
+          <t>R-07、P2-09</t>
+        </is>
+      </c>
+      <c r="I82" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J82" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K82" s="22" t="n"/>
+      <c r="L82" s="20">
         <f>IF(J82="已完成",IF(K82="","",MAX(0,K82-F82)),IF(TODAY()&gt;F82,TODAY()-F82,""))</f>
         <v/>
       </c>
-      <c r="M82" s="24" t="inlineStr"/>
-    </row>
-    <row r="83" ht="34" customHeight="1">
+      <c r="M82" s="21" t="inlineStr"/>
+    </row>
+    <row r="83" ht="19" customHeight="1">
       <c r="A83" s="23" t="n">
         <v>77</v>
       </c>
-      <c r="B83" s="23" t="inlineStr">
-        <is>
-          <t>開發</t>
+      <c r="B83" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
         </is>
       </c>
       <c r="C83" s="24" t="inlineStr">
         <is>
-          <t>出廠模式和工位</t>
+          <t>內部測試</t>
         </is>
       </c>
       <c r="D83" s="24" t="inlineStr">
         <is>
-          <t>工位作業指導書（給工廠工人看）</t>
+          <t>20 台內部測試，每週出一次報表</t>
         </is>
       </c>
       <c r="E83" s="25" t="n">
+        <v>46328</v>
+      </c>
+      <c r="F83" s="25" t="n">
         <v>46353</v>
       </c>
-      <c r="F83" s="25" t="n">
-        <v>46358</v>
-      </c>
       <c r="G83" s="24" t="inlineStr">
         <is>
-          <t>工人照著做就能操作，不用我們在場</t>
+          <t>4 份週報齊全；第 4 週出測試報告</t>
         </is>
       </c>
       <c r="H83" s="24" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-07</t>
         </is>
       </c>
       <c r="I83" s="24" t="inlineStr">
         <is>
-          <t>Jacky</t>
+          <t>全體</t>
         </is>
       </c>
       <c r="J83" s="23" t="inlineStr">
@@ -5770,119 +5778,111 @@
         <f>IF(J83="已完成",IF(K83="","",MAX(0,K83-F83)),IF(TODAY()&gt;F83,TODAY()-F83,""))</f>
         <v/>
       </c>
-      <c r="M83" s="24" t="inlineStr">
-        <is>
-          <t>對接人審閱</t>
-        </is>
-      </c>
+      <c r="M83" s="24" t="inlineStr"/>
     </row>
     <row r="84" ht="34" customHeight="1">
-      <c r="A84" s="23" t="n">
+      <c r="A84" s="20" t="n">
         <v>78</v>
       </c>
-      <c r="B84" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
-        </is>
-      </c>
-      <c r="C84" s="24" t="inlineStr">
+      <c r="B84" s="20" t="inlineStr">
+        <is>
+          <t>開發</t>
+        </is>
+      </c>
+      <c r="C84" s="21" t="inlineStr">
         <is>
           <t>出廠模式和工位</t>
         </is>
       </c>
-      <c r="D84" s="24" t="inlineStr">
-        <is>
-          <t>工位在玩具廠試跑 10 台</t>
-        </is>
-      </c>
-      <c r="E84" s="25" t="n">
-        <v>46357</v>
-      </c>
-      <c r="F84" s="25" t="n">
-        <v>46360</v>
-      </c>
-      <c r="G84" s="24" t="inlineStr">
-        <is>
-          <t>10 台全部通過</t>
-        </is>
-      </c>
-      <c r="H84" s="24" t="inlineStr">
+      <c r="D84" s="21" t="inlineStr">
+        <is>
+          <t>韌體出廠模式：經序列埠寫入密鑰、品牌、款式</t>
+        </is>
+      </c>
+      <c r="E84" s="22" t="n">
+        <v>46342</v>
+      </c>
+      <c r="F84" s="22" t="n">
+        <v>46346</v>
+      </c>
+      <c r="G84" s="21" t="inlineStr">
+        <is>
+          <t>寫入後重新開機，連上該品牌系統</t>
+        </is>
+      </c>
+      <c r="H84" s="21" t="inlineStr">
         <is>
           <t>R-10</t>
         </is>
       </c>
-      <c r="I84" s="24" t="inlineStr">
-        <is>
-          <t>Jacky、對接人</t>
-        </is>
-      </c>
-      <c r="J84" s="23" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K84" s="25" t="n"/>
-      <c r="L84" s="23">
+      <c r="I84" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J84" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K84" s="22" t="n"/>
+      <c r="L84" s="20">
         <f>IF(J84="已完成",IF(K84="","",MAX(0,K84-F84)),IF(TODAY()&gt;F84,TODAY()-F84,""))</f>
         <v/>
       </c>
-      <c r="M84" s="24" t="inlineStr"/>
+      <c r="M84" s="21" t="inlineStr"/>
     </row>
     <row r="85" ht="34" customHeight="1">
-      <c r="A85" s="20" t="n">
+      <c r="A85" s="23" t="n">
         <v>79</v>
       </c>
-      <c r="B85" s="20" t="inlineStr">
+      <c r="B85" s="23" t="inlineStr">
         <is>
           <t>開發</t>
         </is>
       </c>
-      <c r="C85" s="21" t="inlineStr">
-        <is>
-          <t>出廠韌體定版</t>
-        </is>
-      </c>
-      <c r="D85" s="21" t="inlineStr">
-        <is>
-          <t>打包出廠映像（bootloader、分區表、app、Secure Boot 設定），記錄版本號</t>
-        </is>
-      </c>
-      <c r="E85" s="22" t="n">
-        <v>46349</v>
-      </c>
-      <c r="F85" s="22" t="n">
-        <v>46351</v>
-      </c>
-      <c r="G85" s="21" t="inlineStr">
-        <is>
-          <t>包含藍牙配網、加密、按品牌連線、出廠模式四項</t>
-        </is>
-      </c>
-      <c r="H85" s="21" t="inlineStr">
-        <is>
-          <t>R-10、R-21</t>
-        </is>
-      </c>
-      <c r="I85" s="21" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J85" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K85" s="22" t="n"/>
-      <c r="L85" s="20">
+      <c r="C85" s="24" t="inlineStr">
+        <is>
+          <t>出廠模式和工位</t>
+        </is>
+      </c>
+      <c r="D85" s="24" t="inlineStr">
+        <is>
+          <t>韌體自檢指令：喇叭、麥克風、按鍵、燈、Wi-Fi、電池</t>
+        </is>
+      </c>
+      <c r="E85" s="25" t="n">
+        <v>46342</v>
+      </c>
+      <c r="F85" s="25" t="n">
+        <v>46346</v>
+      </c>
+      <c r="G85" s="24" t="inlineStr">
+        <is>
+          <t>每項回傳通過或失敗</t>
+        </is>
+      </c>
+      <c r="H85" s="24" t="inlineStr">
+        <is>
+          <t>R-10</t>
+        </is>
+      </c>
+      <c r="I85" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J85" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K85" s="25" t="n"/>
+      <c r="L85" s="23">
         <f>IF(J85="已完成",IF(K85="","",MAX(0,K85-F85)),IF(TODAY()&gt;F85,TODAY()-F85,""))</f>
         <v/>
       </c>
-      <c r="M85" s="21" t="inlineStr">
-        <is>
-          <t>11/27 交 Spotpear，之後不能改</t>
-        </is>
-      </c>
+      <c r="M85" s="24" t="inlineStr"/>
     </row>
     <row r="86" ht="34" customHeight="1">
       <c r="A86" s="23" t="n">
@@ -5895,23 +5895,23 @@
       </c>
       <c r="C86" s="24" t="inlineStr">
         <is>
-          <t>出廠韌體定版</t>
+          <t>出廠模式和工位</t>
         </is>
       </c>
       <c r="D86" s="24" t="inlineStr">
         <is>
-          <t>寫 Spotpear 燒錄說明：命令、校驗、MAC 清單格式</t>
+          <t>工位腳本：讀 MAC、產生密鑰、寫入、自檢、登記、顯示結果</t>
         </is>
       </c>
       <c r="E86" s="25" t="n">
+        <v>46344</v>
+      </c>
+      <c r="F86" s="25" t="n">
         <v>46350</v>
       </c>
-      <c r="F86" s="25" t="n">
-        <v>46351</v>
-      </c>
       <c r="G86" s="24" t="inlineStr">
         <is>
-          <t>Spotpear 照著做就能燒</t>
+          <t>一條命令完成一台；結果用大字顯示通過或失敗</t>
         </is>
       </c>
       <c r="H86" s="24" t="inlineStr">
@@ -5940,35 +5940,35 @@
       <c r="A87" s="23" t="n">
         <v>81</v>
       </c>
-      <c r="B87" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
+      <c r="B87" s="23" t="inlineStr">
+        <is>
+          <t>開發</t>
         </is>
       </c>
       <c r="C87" s="24" t="inlineStr">
         <is>
-          <t>出廠韌體定版</t>
+          <t>出廠模式和工位</t>
         </is>
       </c>
       <c r="D87" s="24" t="inlineStr">
         <is>
-          <t>我方用 3 片空白板走一次 Spotpear 的燒錄流程</t>
+          <t>每套系統加登記接口（工位專用憑證）</t>
         </is>
       </c>
       <c r="E87" s="25" t="n">
-        <v>46351</v>
+        <v>46346</v>
       </c>
       <c r="F87" s="25" t="n">
-        <v>46352</v>
+        <v>46350</v>
       </c>
       <c r="G87" s="24" t="inlineStr">
         <is>
-          <t>3 片都能開機、過工位、配網、對話</t>
+          <t>只有工位能登記；同一台不能重複登記</t>
         </is>
       </c>
       <c r="H87" s="24" t="inlineStr">
         <is>
-          <t>R-10</t>
+          <t>R-10、R-34</t>
         </is>
       </c>
       <c r="I87" s="24" t="inlineStr">
@@ -5999,23 +5999,23 @@
       </c>
       <c r="C88" s="24" t="inlineStr">
         <is>
-          <t>出廠韌體定版</t>
+          <t>出廠模式和工位</t>
         </is>
       </c>
       <c r="D88" s="24" t="inlineStr">
         <is>
-          <t>Spotpear 試燒 10 片寄回，我方驗證</t>
+          <t>連續 10 台過工位</t>
         </is>
       </c>
       <c r="E88" s="25" t="n">
+        <v>46351</v>
+      </c>
+      <c r="F88" s="25" t="n">
         <v>46353</v>
       </c>
-      <c r="F88" s="25" t="n">
-        <v>46358</v>
-      </c>
       <c r="G88" s="24" t="inlineStr">
         <is>
-          <t>10 片開機、工位寫入、配網、對話、OTA 全部正常</t>
+          <t>10 台全部通過；每台不超過 1.5 分鐘</t>
         </is>
       </c>
       <c r="H88" s="24" t="inlineStr">
@@ -6038,102 +6038,98 @@
         <f>IF(J88="已完成",IF(K88="","",MAX(0,K88-F88)),IF(TODAY()&gt;F88,TODAY()-F88,""))</f>
         <v/>
       </c>
-      <c r="M88" s="24" t="inlineStr">
-        <is>
-          <t>要在 12/4 量產板到廠前驗完</t>
-        </is>
-      </c>
+      <c r="M88" s="24" t="inlineStr"/>
     </row>
     <row r="89" ht="34" customHeight="1">
-      <c r="A89" s="20" t="n">
+      <c r="A89" s="23" t="n">
         <v>83</v>
       </c>
-      <c r="B89" s="20" t="inlineStr">
-        <is>
-          <t>開發</t>
-        </is>
-      </c>
-      <c r="C89" s="21" t="inlineStr">
-        <is>
-          <t>網頁功能凍結</t>
-        </is>
-      </c>
-      <c r="D89" s="21" t="inlineStr">
-        <is>
-          <t>錯誤提示：Wi-Fi 密碼錯、玩具已被綁定、斷網</t>
-        </is>
-      </c>
-      <c r="E89" s="22" t="n">
-        <v>46349</v>
-      </c>
-      <c r="F89" s="22" t="n">
+      <c r="B89" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="C89" s="24" t="inlineStr">
+        <is>
+          <t>出廠模式和工位</t>
+        </is>
+      </c>
+      <c r="D89" s="24" t="inlineStr">
+        <is>
+          <t>混入壞板：拔掉喇叭、拔掉麥克風、低電、重複登記</t>
+        </is>
+      </c>
+      <c r="E89" s="25" t="n">
         <v>46351</v>
       </c>
-      <c r="G89" s="21" t="inlineStr">
-        <is>
-          <t>每種情況都有清楚提示，告訴用戶下一步做什麼</t>
-        </is>
-      </c>
-      <c r="H89" s="21" t="inlineStr">
-        <is>
-          <t>R-28</t>
-        </is>
-      </c>
-      <c r="I89" s="21" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J89" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K89" s="22" t="n"/>
-      <c r="L89" s="20">
+      <c r="F89" s="25" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G89" s="24" t="inlineStr">
+        <is>
+          <t>每種都被攔下並顯示原因</t>
+        </is>
+      </c>
+      <c r="H89" s="24" t="inlineStr">
+        <is>
+          <t>R-10</t>
+        </is>
+      </c>
+      <c r="I89" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J89" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K89" s="25" t="n"/>
+      <c r="L89" s="23">
         <f>IF(J89="已完成",IF(K89="","",MAX(0,K89-F89)),IF(TODAY()&gt;F89,TODAY()-F89,""))</f>
         <v/>
       </c>
-      <c r="M89" s="21" t="inlineStr"/>
+      <c r="M89" s="24" t="inlineStr"/>
     </row>
     <row r="90" ht="34" customHeight="1">
       <c r="A90" s="23" t="n">
         <v>84</v>
       </c>
-      <c r="B90" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
+      <c r="B90" s="23" t="inlineStr">
+        <is>
+          <t>開發</t>
         </is>
       </c>
       <c r="C90" s="24" t="inlineStr">
         <is>
-          <t>網頁功能凍結</t>
+          <t>出廠模式和工位</t>
         </is>
       </c>
       <c r="D90" s="24" t="inlineStr">
         <is>
-          <t>兩個品牌全流程：安裝 → 登入 → 配網 → 綁定 → 對話 → 解綁</t>
+          <t>工位作業指導書（給工廠工人看）</t>
         </is>
       </c>
       <c r="E90" s="25" t="n">
-        <v>46352</v>
+        <v>46353</v>
       </c>
       <c r="F90" s="25" t="n">
-        <v>46353</v>
+        <v>46358</v>
       </c>
       <c r="G90" s="24" t="inlineStr">
         <is>
-          <t>iOS、Android 各兩款手機全部通過</t>
+          <t>工人照著做就能操作，不用我們在場</t>
         </is>
       </c>
       <c r="H90" s="24" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="I90" s="24" t="inlineStr">
         <is>
-          <t>Jacky、Neo</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="J90" s="23" t="inlineStr">
@@ -6146,42 +6142,50 @@
         <f>IF(J90="已完成",IF(K90="","",MAX(0,K90-F90)),IF(TODAY()&gt;F90,TODAY()-F90,""))</f>
         <v/>
       </c>
-      <c r="M90" s="24" t="inlineStr"/>
-    </row>
-    <row r="91" ht="19" customHeight="1">
+      <c r="M90" s="24" t="inlineStr">
+        <is>
+          <t>對接人審閱</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="34" customHeight="1">
       <c r="A91" s="23" t="n">
         <v>85</v>
       </c>
-      <c r="B91" s="23" t="inlineStr">
-        <is>
-          <t>開發</t>
+      <c r="B91" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
         </is>
       </c>
       <c r="C91" s="24" t="inlineStr">
         <is>
-          <t>網頁功能凍結</t>
+          <t>出廠模式和工位</t>
         </is>
       </c>
       <c r="D91" s="24" t="inlineStr">
         <is>
-          <t>功能凍結：開發布分支，之後只修 bug</t>
+          <t>工位在玩具廠試跑 10 台</t>
         </is>
       </c>
       <c r="E91" s="25" t="n">
-        <v>46353</v>
+        <v>46357</v>
       </c>
       <c r="F91" s="25" t="n">
-        <v>46353</v>
+        <v>46360</v>
       </c>
       <c r="G91" s="24" t="inlineStr">
         <is>
-          <t>凍結版本有標籤</t>
-        </is>
-      </c>
-      <c r="H91" s="24" t="inlineStr"/>
+          <t>10 台全部通過</t>
+        </is>
+      </c>
+      <c r="H91" s="24" t="inlineStr">
+        <is>
+          <t>R-10</t>
+        </is>
+      </c>
       <c r="I91" s="24" t="inlineStr">
         <is>
-          <t>Jacky</t>
+          <t>Jacky、對接人</t>
         </is>
       </c>
       <c r="J91" s="23" t="inlineStr">
@@ -6207,28 +6211,28 @@
       </c>
       <c r="C92" s="21" t="inlineStr">
         <is>
-          <t>三套系統</t>
+          <t>出廠韌體定版</t>
         </is>
       </c>
       <c r="D92" s="21" t="inlineStr">
         <is>
-          <t>部署腳本：按品牌逐套更新資料庫、部署、冒煙測試</t>
+          <t>打包出廠映像（bootloader、分區表、app、Secure Boot 設定），記錄版本號</t>
         </is>
       </c>
       <c r="E92" s="22" t="n">
-        <v>46342</v>
+        <v>46349</v>
       </c>
       <c r="F92" s="22" t="n">
-        <v>46350</v>
+        <v>46351</v>
       </c>
       <c r="G92" s="21" t="inlineStr">
         <is>
-          <t>一條命令跑完三套，AI Buddy 先</t>
+          <t>包含藍牙配網、加密、按品牌連線、出廠模式四項</t>
         </is>
       </c>
       <c r="H92" s="21" t="inlineStr">
         <is>
-          <t>R-34</t>
+          <t>R-10、R-21</t>
         </is>
       </c>
       <c r="I92" s="21" t="inlineStr">
@@ -6246,7 +6250,11 @@
         <f>IF(J92="已完成",IF(K92="","",MAX(0,K92-F92)),IF(TODAY()&gt;F92,TODAY()-F92,""))</f>
         <v/>
       </c>
-      <c r="M92" s="21" t="inlineStr"/>
+      <c r="M92" s="21" t="inlineStr">
+        <is>
+          <t>11/27 交 Spotpear，之後不能改</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="34" customHeight="1">
       <c r="A93" s="23" t="n">
@@ -6259,28 +6267,28 @@
       </c>
       <c r="C93" s="24" t="inlineStr">
         <is>
-          <t>三套系統</t>
+          <t>出廠韌體定版</t>
         </is>
       </c>
       <c r="D93" s="24" t="inlineStr">
         <is>
-          <t>開快活、政協青年聯會兩套系統（子網域、密鑰、資料庫、AI 供應商 key）</t>
+          <t>寫 Spotpear 燒錄說明：命令、校驗、MAC 清單格式</t>
         </is>
       </c>
       <c r="E93" s="25" t="n">
-        <v>46349</v>
+        <v>46350</v>
       </c>
       <c r="F93" s="25" t="n">
-        <v>46353</v>
+        <v>46351</v>
       </c>
       <c r="G93" s="24" t="inlineStr">
         <is>
-          <t>兩套都能登入和對話</t>
+          <t>Spotpear 照著做就能燒</t>
         </is>
       </c>
       <c r="H93" s="24" t="inlineStr">
         <is>
-          <t>R-34</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="I93" s="24" t="inlineStr">
@@ -6298,45 +6306,41 @@
         <f>IF(J93="已完成",IF(K93="","",MAX(0,K93-F93)),IF(TODAY()&gt;F93,TODAY()-F93,""))</f>
         <v/>
       </c>
-      <c r="M93" s="24" t="inlineStr">
-        <is>
-          <t>對接人跟客戶確認子網域</t>
-        </is>
-      </c>
+      <c r="M93" s="24" t="inlineStr"/>
     </row>
     <row r="94" ht="34" customHeight="1">
       <c r="A94" s="23" t="n">
         <v>88</v>
       </c>
-      <c r="B94" s="23" t="inlineStr">
-        <is>
-          <t>開發</t>
+      <c r="B94" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
         </is>
       </c>
       <c r="C94" s="24" t="inlineStr">
         <is>
-          <t>三套系統</t>
+          <t>出廠韌體定版</t>
         </is>
       </c>
       <c r="D94" s="24" t="inlineStr">
         <is>
-          <t>每套各自備份；一個監控面板，告警寫明品牌</t>
+          <t>我方用 3 片空白板走一次 Spotpear 的燒錄流程</t>
         </is>
       </c>
       <c r="E94" s="25" t="n">
-        <v>46353</v>
+        <v>46351</v>
       </c>
       <c r="F94" s="25" t="n">
-        <v>46358</v>
+        <v>46352</v>
       </c>
       <c r="G94" s="24" t="inlineStr">
         <is>
-          <t>三套都有每日備份；告警訊息帶品牌名</t>
+          <t>3 片都能開機、過工位、配網、對話</t>
         </is>
       </c>
       <c r="H94" s="24" t="inlineStr">
         <is>
-          <t>P2-06、P2-07</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="I94" s="24" t="inlineStr">
@@ -6356,7 +6360,7 @@
       </c>
       <c r="M94" s="24" t="inlineStr"/>
     </row>
-    <row r="95" ht="19" customHeight="1">
+    <row r="95" ht="34" customHeight="1">
       <c r="A95" s="23" t="n">
         <v>89</v>
       </c>
@@ -6367,28 +6371,28 @@
       </c>
       <c r="C95" s="24" t="inlineStr">
         <is>
-          <t>三套系統</t>
+          <t>出廠韌體定版</t>
         </is>
       </c>
       <c r="D95" s="24" t="inlineStr">
         <is>
-          <t>三套冒煙測試：登入、對話、OTA 檢查</t>
+          <t>Spotpear 試燒 10 片寄回，我方驗證</t>
         </is>
       </c>
       <c r="E95" s="25" t="n">
-        <v>46359</v>
+        <v>46353</v>
       </c>
       <c r="F95" s="25" t="n">
-        <v>46360</v>
+        <v>46358</v>
       </c>
       <c r="G95" s="24" t="inlineStr">
         <is>
-          <t>三套全部通過</t>
+          <t>10 片開機、工位寫入、配網、對話、OTA 全部正常</t>
         </is>
       </c>
       <c r="H95" s="24" t="inlineStr">
         <is>
-          <t>R-34</t>
+          <t>R-10</t>
         </is>
       </c>
       <c r="I95" s="24" t="inlineStr">
@@ -6406,61 +6410,65 @@
         <f>IF(J95="已完成",IF(K95="","",MAX(0,K95-F95)),IF(TODAY()&gt;F95,TODAY()-F95,""))</f>
         <v/>
       </c>
-      <c r="M95" s="24" t="inlineStr"/>
-    </row>
-    <row r="96" ht="19" customHeight="1">
-      <c r="A96" s="23" t="n">
+      <c r="M95" s="24" t="inlineStr">
+        <is>
+          <t>要在 12/4 量產板到廠前驗完</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="34" customHeight="1">
+      <c r="A96" s="20" t="n">
         <v>90</v>
       </c>
-      <c r="B96" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
-        </is>
-      </c>
-      <c r="C96" s="24" t="inlineStr">
-        <is>
-          <t>三套系統</t>
-        </is>
-      </c>
-      <c r="D96" s="24" t="inlineStr">
-        <is>
-          <t>停掉其中一套</t>
-        </is>
-      </c>
-      <c r="E96" s="25" t="n">
-        <v>46359</v>
-      </c>
-      <c r="F96" s="25" t="n">
-        <v>46360</v>
-      </c>
-      <c r="G96" s="24" t="inlineStr">
-        <is>
-          <t>另外兩套照常使用</t>
-        </is>
-      </c>
-      <c r="H96" s="24" t="inlineStr">
-        <is>
-          <t>R-34</t>
-        </is>
-      </c>
-      <c r="I96" s="24" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J96" s="23" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K96" s="25" t="n"/>
-      <c r="L96" s="23">
+      <c r="B96" s="20" t="inlineStr">
+        <is>
+          <t>開發</t>
+        </is>
+      </c>
+      <c r="C96" s="21" t="inlineStr">
+        <is>
+          <t>網頁功能凍結</t>
+        </is>
+      </c>
+      <c r="D96" s="21" t="inlineStr">
+        <is>
+          <t>錯誤提示：Wi-Fi 密碼錯、玩具已被綁定、斷網</t>
+        </is>
+      </c>
+      <c r="E96" s="22" t="n">
+        <v>46349</v>
+      </c>
+      <c r="F96" s="22" t="n">
+        <v>46351</v>
+      </c>
+      <c r="G96" s="21" t="inlineStr">
+        <is>
+          <t>每種情況都有清楚提示，告訴用戶下一步做什麼</t>
+        </is>
+      </c>
+      <c r="H96" s="21" t="inlineStr">
+        <is>
+          <t>R-28</t>
+        </is>
+      </c>
+      <c r="I96" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J96" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K96" s="22" t="n"/>
+      <c r="L96" s="20">
         <f>IF(J96="已完成",IF(K96="","",MAX(0,K96-F96)),IF(TODAY()&gt;F96,TODAY()-F96,""))</f>
         <v/>
       </c>
-      <c r="M96" s="24" t="inlineStr"/>
-    </row>
-    <row r="97" ht="19" customHeight="1">
+      <c r="M96" s="21" t="inlineStr"/>
+    </row>
+    <row r="97" ht="34" customHeight="1">
       <c r="A97" s="23" t="n">
         <v>91</v>
       </c>
@@ -6471,33 +6479,33 @@
       </c>
       <c r="C97" s="24" t="inlineStr">
         <is>
-          <t>三套系統</t>
+          <t>網頁功能凍結</t>
         </is>
       </c>
       <c r="D97" s="24" t="inlineStr">
         <is>
-          <t>每套從備份還原一次</t>
+          <t>兩個品牌全流程：安裝 → 登入 → 配網 → 綁定 → 對話 → 解綁</t>
         </is>
       </c>
       <c r="E97" s="25" t="n">
-        <v>46359</v>
+        <v>46352</v>
       </c>
       <c r="F97" s="25" t="n">
-        <v>46360</v>
+        <v>46353</v>
       </c>
       <c r="G97" s="24" t="inlineStr">
         <is>
-          <t>還原後資料完整</t>
+          <t>iOS、Android 各兩款手機全部通過</t>
         </is>
       </c>
       <c r="H97" s="24" t="inlineStr">
         <is>
-          <t>P2-07</t>
+          <t>R-28</t>
         </is>
       </c>
       <c r="I97" s="24" t="inlineStr">
         <is>
-          <t>Jacky</t>
+          <t>Jacky、Neo</t>
         </is>
       </c>
       <c r="J97" s="23" t="inlineStr">
@@ -6512,143 +6520,139 @@
       </c>
       <c r="M97" s="24" t="inlineStr"/>
     </row>
-    <row r="98" ht="34" customHeight="1">
-      <c r="A98" s="20" t="n">
+    <row r="98" ht="19" customHeight="1">
+      <c r="A98" s="23" t="n">
         <v>92</v>
       </c>
-      <c r="B98" s="20" t="inlineStr">
+      <c r="B98" s="23" t="inlineStr">
         <is>
           <t>開發</t>
         </is>
       </c>
-      <c r="C98" s="21" t="inlineStr">
-        <is>
-          <t>系統測試</t>
-        </is>
-      </c>
-      <c r="D98" s="21" t="inlineStr">
-        <is>
-          <t>壓測腳本：模擬設備同時語音對話</t>
-        </is>
-      </c>
-      <c r="E98" s="22" t="n">
-        <v>46349</v>
-      </c>
-      <c r="F98" s="22" t="n">
+      <c r="C98" s="24" t="inlineStr">
+        <is>
+          <t>網頁功能凍結</t>
+        </is>
+      </c>
+      <c r="D98" s="24" t="inlineStr">
+        <is>
+          <t>功能凍結：開發布分支，之後只修 bug</t>
+        </is>
+      </c>
+      <c r="E98" s="25" t="n">
         <v>46353</v>
       </c>
-      <c r="G98" s="21" t="inlineStr">
-        <is>
-          <t>可以設定同時對話數，輸出首字延遲和錯誤率</t>
-        </is>
-      </c>
-      <c r="H98" s="21" t="inlineStr">
-        <is>
-          <t>P2-08</t>
-        </is>
-      </c>
-      <c r="I98" s="21" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J98" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K98" s="22" t="n"/>
-      <c r="L98" s="20">
+      <c r="F98" s="25" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G98" s="24" t="inlineStr">
+        <is>
+          <t>凍結版本有標籤</t>
+        </is>
+      </c>
+      <c r="H98" s="24" t="inlineStr"/>
+      <c r="I98" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J98" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K98" s="25" t="n"/>
+      <c r="L98" s="23">
         <f>IF(J98="已完成",IF(K98="","",MAX(0,K98-F98)),IF(TODAY()&gt;F98,TODAY()-F98,""))</f>
         <v/>
       </c>
-      <c r="M98" s="21" t="inlineStr"/>
+      <c r="M98" s="24" t="inlineStr"/>
     </row>
     <row r="99" ht="34" customHeight="1">
-      <c r="A99" s="23" t="n">
+      <c r="A99" s="20" t="n">
         <v>93</v>
       </c>
-      <c r="B99" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
-        </is>
-      </c>
-      <c r="C99" s="24" t="inlineStr">
-        <is>
-          <t>系統測試</t>
-        </is>
-      </c>
-      <c r="D99" s="24" t="inlineStr">
-        <is>
-          <t>按 3,000 台規模壓測：150–300 個同時對話</t>
-        </is>
-      </c>
-      <c r="E99" s="25" t="n">
-        <v>46356</v>
-      </c>
-      <c r="F99" s="25" t="n">
-        <v>46359</v>
-      </c>
-      <c r="G99" s="24" t="inlineStr">
-        <is>
-          <t>首字延遲和錯誤率在目標內；伺服器不崩潰</t>
-        </is>
-      </c>
-      <c r="H99" s="24" t="inlineStr">
-        <is>
-          <t>P2-08</t>
-        </is>
-      </c>
-      <c r="I99" s="24" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J99" s="23" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K99" s="25" t="n"/>
-      <c r="L99" s="23">
+      <c r="B99" s="20" t="inlineStr">
+        <is>
+          <t>開發</t>
+        </is>
+      </c>
+      <c r="C99" s="21" t="inlineStr">
+        <is>
+          <t>三套系統</t>
+        </is>
+      </c>
+      <c r="D99" s="21" t="inlineStr">
+        <is>
+          <t>部署腳本：按品牌逐套更新資料庫、部署、冒煙測試</t>
+        </is>
+      </c>
+      <c r="E99" s="22" t="n">
+        <v>46342</v>
+      </c>
+      <c r="F99" s="22" t="n">
+        <v>46350</v>
+      </c>
+      <c r="G99" s="21" t="inlineStr">
+        <is>
+          <t>一條命令跑完三套，AI Buddy 先</t>
+        </is>
+      </c>
+      <c r="H99" s="21" t="inlineStr">
+        <is>
+          <t>R-34</t>
+        </is>
+      </c>
+      <c r="I99" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J99" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K99" s="22" t="n"/>
+      <c r="L99" s="20">
         <f>IF(J99="已完成",IF(K99="","",MAX(0,K99-F99)),IF(TODAY()&gt;F99,TODAY()-F99,""))</f>
         <v/>
       </c>
-      <c r="M99" s="24" t="inlineStr"/>
+      <c r="M99" s="21" t="inlineStr"/>
     </row>
     <row r="100" ht="34" customHeight="1">
       <c r="A100" s="23" t="n">
         <v>94</v>
       </c>
-      <c r="B100" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
+      <c r="B100" s="23" t="inlineStr">
+        <is>
+          <t>開發</t>
         </is>
       </c>
       <c r="C100" s="24" t="inlineStr">
         <is>
-          <t>系統測試</t>
+          <t>三套系統</t>
         </is>
       </c>
       <c r="D100" s="24" t="inlineStr">
         <is>
-          <t>安全測試：三套系統各重跑一次 P0 檢查</t>
+          <t>開快活、政協青年聯會兩套系統（子網域、密鑰、資料庫、AI 供應商 key）</t>
         </is>
       </c>
       <c r="E100" s="25" t="n">
-        <v>46356</v>
+        <v>46349</v>
       </c>
       <c r="F100" s="25" t="n">
-        <v>46360</v>
+        <v>46353</v>
       </c>
       <c r="G100" s="24" t="inlineStr">
         <is>
-          <t>未登入讀不到資料；未認領設備被拒；管理員權限正確</t>
+          <t>兩套都能登入和對話</t>
         </is>
       </c>
       <c r="H100" s="24" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>R-34</t>
         </is>
       </c>
       <c r="I100" s="24" t="inlineStr">
@@ -6666,46 +6670,50 @@
         <f>IF(J100="已完成",IF(K100="","",MAX(0,K100-F100)),IF(TODAY()&gt;F100,TODAY()-F100,""))</f>
         <v/>
       </c>
-      <c r="M100" s="24" t="inlineStr"/>
+      <c r="M100" s="24" t="inlineStr">
+        <is>
+          <t>對接人跟客戶確認子網域</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="34" customHeight="1">
       <c r="A101" s="23" t="n">
         <v>95</v>
       </c>
-      <c r="B101" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
+      <c r="B101" s="23" t="inlineStr">
+        <is>
+          <t>開發</t>
         </is>
       </c>
       <c r="C101" s="24" t="inlineStr">
         <is>
-          <t>系統測試</t>
+          <t>三套系統</t>
         </is>
       </c>
       <c r="D101" s="24" t="inlineStr">
         <is>
-          <t>手機端全流程回歸</t>
+          <t>每套各自備份；一個監控面板，告警寫明品牌</t>
         </is>
       </c>
       <c r="E101" s="25" t="n">
-        <v>46356</v>
+        <v>46353</v>
       </c>
       <c r="F101" s="25" t="n">
-        <v>46360</v>
+        <v>46358</v>
       </c>
       <c r="G101" s="24" t="inlineStr">
         <is>
-          <t>iOS、Android 各兩款全部通過；嚴重問題 0 個</t>
+          <t>三套都有每日備份；告警訊息帶品牌名</t>
         </is>
       </c>
       <c r="H101" s="24" t="inlineStr">
         <is>
-          <t>R-28</t>
+          <t>P2-06、P2-07</t>
         </is>
       </c>
       <c r="I101" s="24" t="inlineStr">
         <is>
-          <t>Neo</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="J101" s="23" t="inlineStr">
@@ -6718,63 +6726,59 @@
         <f>IF(J101="已完成",IF(K101="","",MAX(0,K101-F101)),IF(TODAY()&gt;F101,TODAY()-F101,""))</f>
         <v/>
       </c>
-      <c r="M101" s="24" t="inlineStr">
-        <is>
-          <t>Jacky 修問題</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="34" customHeight="1">
-      <c r="A102" s="20" t="n">
+      <c r="M101" s="24" t="inlineStr"/>
+    </row>
+    <row r="102" ht="19" customHeight="1">
+      <c r="A102" s="23" t="n">
         <v>96</v>
       </c>
-      <c r="B102" s="20" t="inlineStr">
-        <is>
-          <t>開發</t>
-        </is>
-      </c>
-      <c r="C102" s="21" t="inlineStr">
-        <is>
-          <t>首次 OTA 版本</t>
-        </is>
-      </c>
-      <c r="D102" s="21" t="inlineStr">
-        <is>
-          <t>首次開機 OTA 版本定版（出廠後的修正和新功能）</t>
-        </is>
-      </c>
-      <c r="E102" s="22" t="n">
-        <v>46363</v>
-      </c>
-      <c r="F102" s="22" t="n">
-        <v>46367</v>
-      </c>
-      <c r="G102" s="21" t="inlineStr">
-        <is>
-          <t>版本號記錄好；發佈到三套系統</t>
-        </is>
-      </c>
-      <c r="H102" s="21" t="inlineStr">
-        <is>
-          <t>P0-13</t>
-        </is>
-      </c>
-      <c r="I102" s="21" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J102" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K102" s="22" t="n"/>
-      <c r="L102" s="20">
+      <c r="B102" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="C102" s="24" t="inlineStr">
+        <is>
+          <t>三套系統</t>
+        </is>
+      </c>
+      <c r="D102" s="24" t="inlineStr">
+        <is>
+          <t>三套冒煙測試：登入、對話、OTA 檢查</t>
+        </is>
+      </c>
+      <c r="E102" s="25" t="n">
+        <v>46359</v>
+      </c>
+      <c r="F102" s="25" t="n">
+        <v>46360</v>
+      </c>
+      <c r="G102" s="24" t="inlineStr">
+        <is>
+          <t>三套全部通過</t>
+        </is>
+      </c>
+      <c r="H102" s="24" t="inlineStr">
+        <is>
+          <t>R-34</t>
+        </is>
+      </c>
+      <c r="I102" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J102" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K102" s="25" t="n"/>
+      <c r="L102" s="23">
         <f>IF(J102="已完成",IF(K102="","",MAX(0,K102-F102)),IF(TODAY()&gt;F102,TODAY()-F102,""))</f>
         <v/>
       </c>
-      <c r="M102" s="21" t="inlineStr"/>
+      <c r="M102" s="24" t="inlineStr"/>
     </row>
     <row r="103" ht="19" customHeight="1">
       <c r="A103" s="23" t="n">
@@ -6787,28 +6791,28 @@
       </c>
       <c r="C103" s="24" t="inlineStr">
         <is>
-          <t>首次 OTA 版本</t>
+          <t>三套系統</t>
         </is>
       </c>
       <c r="D103" s="24" t="inlineStr">
         <is>
-          <t>出廠韌體升級到這個版本，再回滾</t>
+          <t>停掉其中一套</t>
         </is>
       </c>
       <c r="E103" s="25" t="n">
-        <v>46366</v>
+        <v>46359</v>
       </c>
       <c r="F103" s="25" t="n">
-        <v>46367</v>
+        <v>46360</v>
       </c>
       <c r="G103" s="24" t="inlineStr">
         <is>
-          <t>升級和回滾都成功</t>
+          <t>另外兩套照常使用</t>
         </is>
       </c>
       <c r="H103" s="24" t="inlineStr">
         <is>
-          <t>P0-13</t>
+          <t>R-34</t>
         </is>
       </c>
       <c r="I103" s="24" t="inlineStr">
@@ -6828,109 +6832,109 @@
       </c>
       <c r="M103" s="24" t="inlineStr"/>
     </row>
-    <row r="104" ht="34" customHeight="1">
-      <c r="A104" s="20" t="n">
+    <row r="104" ht="19" customHeight="1">
+      <c r="A104" s="23" t="n">
         <v>98</v>
       </c>
-      <c r="B104" s="20" t="inlineStr">
+      <c r="B104" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="C104" s="24" t="inlineStr">
+        <is>
+          <t>三套系統</t>
+        </is>
+      </c>
+      <c r="D104" s="24" t="inlineStr">
+        <is>
+          <t>每套從備份還原一次</t>
+        </is>
+      </c>
+      <c r="E104" s="25" t="n">
+        <v>46359</v>
+      </c>
+      <c r="F104" s="25" t="n">
+        <v>46360</v>
+      </c>
+      <c r="G104" s="24" t="inlineStr">
+        <is>
+          <t>還原後資料完整</t>
+        </is>
+      </c>
+      <c r="H104" s="24" t="inlineStr">
+        <is>
+          <t>P2-07</t>
+        </is>
+      </c>
+      <c r="I104" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J104" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K104" s="25" t="n"/>
+      <c r="L104" s="23">
+        <f>IF(J104="已完成",IF(K104="","",MAX(0,K104-F104)),IF(TODAY()&gt;F104,TODAY()-F104,""))</f>
+        <v/>
+      </c>
+      <c r="M104" s="24" t="inlineStr"/>
+    </row>
+    <row r="105" ht="34" customHeight="1">
+      <c r="A105" s="20" t="n">
+        <v>99</v>
+      </c>
+      <c r="B105" s="20" t="inlineStr">
         <is>
           <t>開發</t>
         </is>
       </c>
-      <c r="C104" s="21" t="inlineStr">
-        <is>
-          <t>UAT</t>
-        </is>
-      </c>
-      <c r="D104" s="21" t="inlineStr">
-        <is>
-          <t>UAT 清單：客戶要逐項測的內容</t>
-        </is>
-      </c>
-      <c r="E104" s="22" t="n">
-        <v>46356</v>
-      </c>
-      <c r="F104" s="22" t="n">
-        <v>46360</v>
-      </c>
-      <c r="G104" s="21" t="inlineStr">
-        <is>
-          <t>對接人和客戶確認清單</t>
-        </is>
-      </c>
-      <c r="H104" s="21" t="inlineStr">
-        <is>
-          <t>R-06</t>
-        </is>
-      </c>
-      <c r="I104" s="21" t="inlineStr">
-        <is>
-          <t>Jacky、對接人</t>
-        </is>
-      </c>
-      <c r="J104" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K104" s="22" t="n"/>
-      <c r="L104" s="20">
-        <f>IF(J104="已完成",IF(K104="","",MAX(0,K104-F104)),IF(TODAY()&gt;F104,TODAY()-F104,""))</f>
-        <v/>
-      </c>
-      <c r="M104" s="21" t="inlineStr"/>
-    </row>
-    <row r="105" ht="34" customHeight="1">
-      <c r="A105" s="23" t="n">
-        <v>99</v>
-      </c>
-      <c r="B105" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
-        </is>
-      </c>
-      <c r="C105" s="24" t="inlineStr">
-        <is>
-          <t>UAT</t>
-        </is>
-      </c>
-      <c r="D105" s="24" t="inlineStr">
-        <is>
-          <t>支援客戶 UAT：記錄問題、修復</t>
-        </is>
-      </c>
-      <c r="E105" s="25" t="n">
-        <v>46363</v>
-      </c>
-      <c r="F105" s="25" t="n">
-        <v>46374</v>
-      </c>
-      <c r="G105" s="24" t="inlineStr">
-        <is>
-          <t>客戶書面簽收；嚴重問題 0 個，其他問題都有處理日期</t>
-        </is>
-      </c>
-      <c r="H105" s="24" t="inlineStr">
-        <is>
-          <t>R-06</t>
-        </is>
-      </c>
-      <c r="I105" s="24" t="inlineStr">
-        <is>
-          <t>Jacky、Neo</t>
-        </is>
-      </c>
-      <c r="J105" s="23" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K105" s="25" t="n"/>
-      <c r="L105" s="23">
+      <c r="C105" s="21" t="inlineStr">
+        <is>
+          <t>系統測試</t>
+        </is>
+      </c>
+      <c r="D105" s="21" t="inlineStr">
+        <is>
+          <t>壓測腳本：模擬設備同時語音對話</t>
+        </is>
+      </c>
+      <c r="E105" s="22" t="n">
+        <v>46349</v>
+      </c>
+      <c r="F105" s="22" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G105" s="21" t="inlineStr">
+        <is>
+          <t>可以設定同時對話數，輸出首字延遲和錯誤率</t>
+        </is>
+      </c>
+      <c r="H105" s="21" t="inlineStr">
+        <is>
+          <t>P2-08</t>
+        </is>
+      </c>
+      <c r="I105" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J105" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K105" s="22" t="n"/>
+      <c r="L105" s="20">
         <f>IF(J105="已完成",IF(K105="","",MAX(0,K105-F105)),IF(TODAY()&gt;F105,TODAY()-F105,""))</f>
         <v/>
       </c>
-      <c r="M105" s="24" t="inlineStr"/>
+      <c r="M105" s="21" t="inlineStr"/>
     </row>
     <row r="106" ht="34" customHeight="1">
       <c r="A106" s="23" t="n">
@@ -6943,33 +6947,33 @@
       </c>
       <c r="C106" s="24" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>系統測試</t>
         </is>
       </c>
       <c r="D106" s="24" t="inlineStr">
         <is>
-          <t>3 位非團隊成員從開箱到第一次對話</t>
+          <t>按 3,000 台規模壓測：150–300 個同時對話</t>
         </is>
       </c>
       <c r="E106" s="25" t="n">
-        <v>46370</v>
+        <v>46356</v>
       </c>
       <c r="F106" s="25" t="n">
-        <v>46374</v>
+        <v>46359</v>
       </c>
       <c r="G106" s="24" t="inlineStr">
         <is>
-          <t>3 人都在 10 分鐘內完成</t>
+          <t>首字延遲和錯誤率在目標內；伺服器不崩潰</t>
         </is>
       </c>
       <c r="H106" s="24" t="inlineStr">
         <is>
-          <t>R-06</t>
+          <t>P2-08</t>
         </is>
       </c>
       <c r="I106" s="24" t="inlineStr">
         <is>
-          <t>對接人</t>
+          <t>Jacky</t>
         </is>
       </c>
       <c r="J106" s="23" t="inlineStr">
@@ -6982,94 +6986,98 @@
         <f>IF(J106="已完成",IF(K106="","",MAX(0,K106-F106)),IF(TODAY()&gt;F106,TODAY()-F106,""))</f>
         <v/>
       </c>
-      <c r="M106" s="24" t="inlineStr">
-        <is>
-          <t>Jacky 在旁記錄卡住的地方</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="19" customHeight="1">
-      <c r="A107" s="20" t="n">
+      <c r="M106" s="24" t="inlineStr"/>
+    </row>
+    <row r="107" ht="34" customHeight="1">
+      <c r="A107" s="23" t="n">
         <v>101</v>
       </c>
-      <c r="B107" s="27" t="inlineStr">
+      <c r="B107" s="26" t="inlineStr">
         <is>
           <t>測試</t>
         </is>
       </c>
-      <c r="C107" s="21" t="inlineStr">
-        <is>
-          <t>上線前確認</t>
-        </is>
-      </c>
-      <c r="D107" s="21" t="inlineStr">
-        <is>
-          <t>UAT 遺留問題逐項複測</t>
-        </is>
-      </c>
-      <c r="E107" s="22" t="n">
-        <v>46391</v>
-      </c>
-      <c r="F107" s="22" t="n">
-        <v>46395</v>
-      </c>
-      <c r="G107" s="21" t="inlineStr">
-        <is>
-          <t>全部處理完</t>
-        </is>
-      </c>
-      <c r="H107" s="21" t="inlineStr"/>
-      <c r="I107" s="21" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J107" s="20" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K107" s="22" t="n"/>
-      <c r="L107" s="20">
+      <c r="C107" s="24" t="inlineStr">
+        <is>
+          <t>系統測試</t>
+        </is>
+      </c>
+      <c r="D107" s="24" t="inlineStr">
+        <is>
+          <t>安全測試：三套系統各重跑一次 P0 檢查</t>
+        </is>
+      </c>
+      <c r="E107" s="25" t="n">
+        <v>46356</v>
+      </c>
+      <c r="F107" s="25" t="n">
+        <v>46360</v>
+      </c>
+      <c r="G107" s="24" t="inlineStr">
+        <is>
+          <t>未登入讀不到資料；未認領設備被拒；管理員權限正確</t>
+        </is>
+      </c>
+      <c r="H107" s="24" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I107" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J107" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K107" s="25" t="n"/>
+      <c r="L107" s="23">
         <f>IF(J107="已完成",IF(K107="","",MAX(0,K107-F107)),IF(TODAY()&gt;F107,TODAY()-F107,""))</f>
         <v/>
       </c>
-      <c r="M107" s="21" t="inlineStr"/>
-    </row>
-    <row r="108" ht="19" customHeight="1">
+      <c r="M107" s="24" t="inlineStr"/>
+    </row>
+    <row r="108" ht="34" customHeight="1">
       <c r="A108" s="23" t="n">
         <v>102</v>
       </c>
-      <c r="B108" s="23" t="inlineStr">
-        <is>
-          <t>開發</t>
+      <c r="B108" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
         </is>
       </c>
       <c r="C108" s="24" t="inlineStr">
         <is>
-          <t>上線前確認</t>
+          <t>系統測試</t>
         </is>
       </c>
       <c r="D108" s="24" t="inlineStr">
         <is>
-          <t>正式環境凍結，只修 bug</t>
+          <t>手機端全流程回歸</t>
         </is>
       </c>
       <c r="E108" s="25" t="n">
-        <v>46395</v>
+        <v>46356</v>
       </c>
       <c r="F108" s="25" t="n">
-        <v>46395</v>
+        <v>46360</v>
       </c>
       <c r="G108" s="24" t="inlineStr">
         <is>
-          <t>凍結版本有標籤</t>
-        </is>
-      </c>
-      <c r="H108" s="24" t="inlineStr"/>
+          <t>iOS、Android 各兩款全部通過；嚴重問題 0 個</t>
+        </is>
+      </c>
+      <c r="H108" s="24" t="inlineStr">
+        <is>
+          <t>R-28</t>
+        </is>
+      </c>
       <c r="I108" s="24" t="inlineStr">
         <is>
-          <t>Jacky</t>
+          <t>Neo</t>
         </is>
       </c>
       <c r="J108" s="23" t="inlineStr">
@@ -7082,61 +7090,65 @@
         <f>IF(J108="已完成",IF(K108="","",MAX(0,K108-F108)),IF(TODAY()&gt;F108,TODAY()-F108,""))</f>
         <v/>
       </c>
-      <c r="M108" s="24" t="inlineStr"/>
-    </row>
-    <row r="109" ht="19" customHeight="1">
-      <c r="A109" s="23" t="n">
+      <c r="M108" s="24" t="inlineStr">
+        <is>
+          <t>Jacky 修問題</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="34" customHeight="1">
+      <c r="A109" s="20" t="n">
         <v>103</v>
       </c>
-      <c r="B109" s="26" t="inlineStr">
-        <is>
-          <t>測試</t>
-        </is>
-      </c>
-      <c r="C109" s="24" t="inlineStr">
-        <is>
-          <t>上線前確認</t>
-        </is>
-      </c>
-      <c r="D109" s="24" t="inlineStr">
-        <is>
-          <t>每套系統觸發一次告警</t>
-        </is>
-      </c>
-      <c r="E109" s="25" t="n">
-        <v>46391</v>
-      </c>
-      <c r="F109" s="25" t="n">
-        <v>46395</v>
-      </c>
-      <c r="G109" s="24" t="inlineStr">
-        <is>
-          <t>告警送到並寫明品牌</t>
-        </is>
-      </c>
-      <c r="H109" s="24" t="inlineStr">
-        <is>
-          <t>P2-06</t>
-        </is>
-      </c>
-      <c r="I109" s="24" t="inlineStr">
-        <is>
-          <t>Jacky</t>
-        </is>
-      </c>
-      <c r="J109" s="23" t="inlineStr">
-        <is>
-          <t>未開始</t>
-        </is>
-      </c>
-      <c r="K109" s="25" t="n"/>
-      <c r="L109" s="23">
+      <c r="B109" s="20" t="inlineStr">
+        <is>
+          <t>開發</t>
+        </is>
+      </c>
+      <c r="C109" s="21" t="inlineStr">
+        <is>
+          <t>首次 OTA 版本</t>
+        </is>
+      </c>
+      <c r="D109" s="21" t="inlineStr">
+        <is>
+          <t>首次開機 OTA 版本定版（出廠後的修正和新功能）</t>
+        </is>
+      </c>
+      <c r="E109" s="22" t="n">
+        <v>46363</v>
+      </c>
+      <c r="F109" s="22" t="n">
+        <v>46367</v>
+      </c>
+      <c r="G109" s="21" t="inlineStr">
+        <is>
+          <t>版本號記錄好；發佈到三套系統</t>
+        </is>
+      </c>
+      <c r="H109" s="21" t="inlineStr">
+        <is>
+          <t>P0-13</t>
+        </is>
+      </c>
+      <c r="I109" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J109" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K109" s="22" t="n"/>
+      <c r="L109" s="20">
         <f>IF(J109="已完成",IF(K109="","",MAX(0,K109-F109)),IF(TODAY()&gt;F109,TODAY()-F109,""))</f>
         <v/>
       </c>
-      <c r="M109" s="24" t="inlineStr"/>
-    </row>
-    <row r="110" ht="34" customHeight="1">
+      <c r="M109" s="21" t="inlineStr"/>
+    </row>
+    <row r="110" ht="19" customHeight="1">
       <c r="A110" s="23" t="n">
         <v>104</v>
       </c>
@@ -7147,28 +7159,28 @@
       </c>
       <c r="C110" s="24" t="inlineStr">
         <is>
-          <t>上線前確認</t>
+          <t>首次 OTA 版本</t>
         </is>
       </c>
       <c r="D110" s="24" t="inlineStr">
         <is>
-          <t>對照出貨 MAC 清單，檢查設備登記</t>
+          <t>出廠韌體升級到這個版本，再回滾</t>
         </is>
       </c>
       <c r="E110" s="25" t="n">
-        <v>46398</v>
+        <v>46366</v>
       </c>
       <c r="F110" s="25" t="n">
-        <v>46402</v>
+        <v>46367</v>
       </c>
       <c r="G110" s="24" t="inlineStr">
         <is>
-          <t>每台都已在對應品牌的系統登記</t>
+          <t>升級和回滾都成功</t>
         </is>
       </c>
       <c r="H110" s="24" t="inlineStr">
         <is>
-          <t>R-10、R-15</t>
+          <t>P0-13</t>
         </is>
       </c>
       <c r="I110" s="24" t="inlineStr">
@@ -7188,52 +7200,412 @@
       </c>
       <c r="M110" s="24" t="inlineStr"/>
     </row>
-    <row r="112">
-      <c r="A112" s="12" t="inlineStr">
+    <row r="111" ht="34" customHeight="1">
+      <c r="A111" s="20" t="n">
+        <v>105</v>
+      </c>
+      <c r="B111" s="20" t="inlineStr">
+        <is>
+          <t>開發</t>
+        </is>
+      </c>
+      <c r="C111" s="21" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="D111" s="21" t="inlineStr">
+        <is>
+          <t>UAT 清單：客戶要逐項測的內容</t>
+        </is>
+      </c>
+      <c r="E111" s="22" t="n">
+        <v>46356</v>
+      </c>
+      <c r="F111" s="22" t="n">
+        <v>46360</v>
+      </c>
+      <c r="G111" s="21" t="inlineStr">
+        <is>
+          <t>對接人和客戶確認清單</t>
+        </is>
+      </c>
+      <c r="H111" s="21" t="inlineStr">
+        <is>
+          <t>R-06</t>
+        </is>
+      </c>
+      <c r="I111" s="21" t="inlineStr">
+        <is>
+          <t>Jacky、對接人</t>
+        </is>
+      </c>
+      <c r="J111" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K111" s="22" t="n"/>
+      <c r="L111" s="20">
+        <f>IF(J111="已完成",IF(K111="","",MAX(0,K111-F111)),IF(TODAY()&gt;F111,TODAY()-F111,""))</f>
+        <v/>
+      </c>
+      <c r="M111" s="21" t="inlineStr"/>
+    </row>
+    <row r="112" ht="34" customHeight="1">
+      <c r="A112" s="23" t="n">
+        <v>106</v>
+      </c>
+      <c r="B112" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="C112" s="24" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="D112" s="24" t="inlineStr">
+        <is>
+          <t>支援客戶 UAT：記錄問題、修復</t>
+        </is>
+      </c>
+      <c r="E112" s="25" t="n">
+        <v>46363</v>
+      </c>
+      <c r="F112" s="25" t="n">
+        <v>46374</v>
+      </c>
+      <c r="G112" s="24" t="inlineStr">
+        <is>
+          <t>客戶書面簽收；嚴重問題 0 個，其他問題都有處理日期</t>
+        </is>
+      </c>
+      <c r="H112" s="24" t="inlineStr">
+        <is>
+          <t>R-06</t>
+        </is>
+      </c>
+      <c r="I112" s="24" t="inlineStr">
+        <is>
+          <t>Jacky、Neo</t>
+        </is>
+      </c>
+      <c r="J112" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K112" s="25" t="n"/>
+      <c r="L112" s="23">
+        <f>IF(J112="已完成",IF(K112="","",MAX(0,K112-F112)),IF(TODAY()&gt;F112,TODAY()-F112,""))</f>
+        <v/>
+      </c>
+      <c r="M112" s="24" t="inlineStr"/>
+    </row>
+    <row r="113" ht="34" customHeight="1">
+      <c r="A113" s="23" t="n">
+        <v>107</v>
+      </c>
+      <c r="B113" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="C113" s="24" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="D113" s="24" t="inlineStr">
+        <is>
+          <t>3 位非團隊成員從開箱到第一次對話</t>
+        </is>
+      </c>
+      <c r="E113" s="25" t="n">
+        <v>46370</v>
+      </c>
+      <c r="F113" s="25" t="n">
+        <v>46374</v>
+      </c>
+      <c r="G113" s="24" t="inlineStr">
+        <is>
+          <t>3 人都在 10 分鐘內完成</t>
+        </is>
+      </c>
+      <c r="H113" s="24" t="inlineStr">
+        <is>
+          <t>R-06</t>
+        </is>
+      </c>
+      <c r="I113" s="24" t="inlineStr">
+        <is>
+          <t>對接人</t>
+        </is>
+      </c>
+      <c r="J113" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K113" s="25" t="n"/>
+      <c r="L113" s="23">
+        <f>IF(J113="已完成",IF(K113="","",MAX(0,K113-F113)),IF(TODAY()&gt;F113,TODAY()-F113,""))</f>
+        <v/>
+      </c>
+      <c r="M113" s="24" t="inlineStr">
+        <is>
+          <t>Jacky 在旁記錄卡住的地方</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="19" customHeight="1">
+      <c r="A114" s="20" t="n">
+        <v>108</v>
+      </c>
+      <c r="B114" s="27" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="C114" s="21" t="inlineStr">
+        <is>
+          <t>上線前確認</t>
+        </is>
+      </c>
+      <c r="D114" s="21" t="inlineStr">
+        <is>
+          <t>UAT 遺留問題逐項複測</t>
+        </is>
+      </c>
+      <c r="E114" s="22" t="n">
+        <v>46391</v>
+      </c>
+      <c r="F114" s="22" t="n">
+        <v>46395</v>
+      </c>
+      <c r="G114" s="21" t="inlineStr">
+        <is>
+          <t>全部處理完</t>
+        </is>
+      </c>
+      <c r="H114" s="21" t="inlineStr"/>
+      <c r="I114" s="21" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J114" s="20" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K114" s="22" t="n"/>
+      <c r="L114" s="20">
+        <f>IF(J114="已完成",IF(K114="","",MAX(0,K114-F114)),IF(TODAY()&gt;F114,TODAY()-F114,""))</f>
+        <v/>
+      </c>
+      <c r="M114" s="21" t="inlineStr"/>
+    </row>
+    <row r="115" ht="19" customHeight="1">
+      <c r="A115" s="23" t="n">
+        <v>109</v>
+      </c>
+      <c r="B115" s="23" t="inlineStr">
+        <is>
+          <t>開發</t>
+        </is>
+      </c>
+      <c r="C115" s="24" t="inlineStr">
+        <is>
+          <t>上線前確認</t>
+        </is>
+      </c>
+      <c r="D115" s="24" t="inlineStr">
+        <is>
+          <t>正式環境凍結，只修 bug</t>
+        </is>
+      </c>
+      <c r="E115" s="25" t="n">
+        <v>46395</v>
+      </c>
+      <c r="F115" s="25" t="n">
+        <v>46395</v>
+      </c>
+      <c r="G115" s="24" t="inlineStr">
+        <is>
+          <t>凍結版本有標籤</t>
+        </is>
+      </c>
+      <c r="H115" s="24" t="inlineStr"/>
+      <c r="I115" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J115" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K115" s="25" t="n"/>
+      <c r="L115" s="23">
+        <f>IF(J115="已完成",IF(K115="","",MAX(0,K115-F115)),IF(TODAY()&gt;F115,TODAY()-F115,""))</f>
+        <v/>
+      </c>
+      <c r="M115" s="24" t="inlineStr"/>
+    </row>
+    <row r="116" ht="19" customHeight="1">
+      <c r="A116" s="23" t="n">
+        <v>110</v>
+      </c>
+      <c r="B116" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="C116" s="24" t="inlineStr">
+        <is>
+          <t>上線前確認</t>
+        </is>
+      </c>
+      <c r="D116" s="24" t="inlineStr">
+        <is>
+          <t>每套系統觸發一次告警</t>
+        </is>
+      </c>
+      <c r="E116" s="25" t="n">
+        <v>46391</v>
+      </c>
+      <c r="F116" s="25" t="n">
+        <v>46395</v>
+      </c>
+      <c r="G116" s="24" t="inlineStr">
+        <is>
+          <t>告警送到並寫明品牌</t>
+        </is>
+      </c>
+      <c r="H116" s="24" t="inlineStr">
+        <is>
+          <t>P2-06</t>
+        </is>
+      </c>
+      <c r="I116" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J116" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K116" s="25" t="n"/>
+      <c r="L116" s="23">
+        <f>IF(J116="已完成",IF(K116="","",MAX(0,K116-F116)),IF(TODAY()&gt;F116,TODAY()-F116,""))</f>
+        <v/>
+      </c>
+      <c r="M116" s="24" t="inlineStr"/>
+    </row>
+    <row r="117" ht="34" customHeight="1">
+      <c r="A117" s="23" t="n">
+        <v>111</v>
+      </c>
+      <c r="B117" s="26" t="inlineStr">
+        <is>
+          <t>測試</t>
+        </is>
+      </c>
+      <c r="C117" s="24" t="inlineStr">
+        <is>
+          <t>上線前確認</t>
+        </is>
+      </c>
+      <c r="D117" s="24" t="inlineStr">
+        <is>
+          <t>對照出貨 MAC 清單，檢查設備登記</t>
+        </is>
+      </c>
+      <c r="E117" s="25" t="n">
+        <v>46398</v>
+      </c>
+      <c r="F117" s="25" t="n">
+        <v>46402</v>
+      </c>
+      <c r="G117" s="24" t="inlineStr">
+        <is>
+          <t>每台都已在對應品牌的系統登記</t>
+        </is>
+      </c>
+      <c r="H117" s="24" t="inlineStr">
+        <is>
+          <t>R-10、R-15</t>
+        </is>
+      </c>
+      <c r="I117" s="24" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
+      <c r="J117" s="23" t="inlineStr">
+        <is>
+          <t>未開始</t>
+        </is>
+      </c>
+      <c r="K117" s="25" t="n"/>
+      <c r="L117" s="23">
+        <f>IF(J117="已完成",IF(K117="","",MAX(0,K117-F117)),IF(TODAY()&gt;F117,TODAY()-F117,""))</f>
+        <v/>
+      </c>
+      <c r="M117" s="24" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="12" t="inlineStr">
         <is>
           <t>說明</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="18" customHeight="1">
-      <c r="A113" s="16" t="inlineStr">
+    <row r="120" ht="18" customHeight="1">
+      <c r="A120" s="16" t="inlineStr">
         <is>
           <t>類型：開發 = 寫程式或做出東西；測試（藍字）= 按「怎樣算完成」實際測過。每個開發工作線最後都有測試項目，測試通過才算這條線完成。</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="18" customHeight="1">
-      <c r="A114" s="16" t="inlineStr">
+    <row r="121" ht="18" customHeight="1">
+      <c r="A121" s="16" t="inlineStr">
         <is>
           <t>黃色底 = 本週到期但未完成。「逾期（天）」由公式計算：未完成且已過完成日，顯示逾期天數；已完成則顯示比計劃晚了幾天。</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="18" customHeight="1">
-      <c r="A115" s="16" t="inlineStr">
+    <row r="122" ht="18" customHeight="1">
+      <c r="A122" s="16" t="inlineStr">
         <is>
           <t>可以用標題列的篩選按鈕只看「開發」或「測試」，或按「完成」排序看到期順序。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:M110"/>
+  <autoFilter ref="A6:M117"/>
   <mergeCells count="8">
     <mergeCell ref="K4:M4"/>
     <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A120:M120"/>
     <mergeCell ref="H4:J4"/>
+    <mergeCell ref="A122:M122"/>
     <mergeCell ref="E4:G4"/>
-    <mergeCell ref="A114:M114"/>
-    <mergeCell ref="A113:M113"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A115:M115"/>
+    <mergeCell ref="A121:M121"/>
   </mergeCells>
-  <conditionalFormatting sqref="A7:M110">
+  <conditionalFormatting sqref="A7:M117">
     <cfRule type="expression" priority="1" dxfId="6">
       <formula>AND($J7&lt;&gt;"已完成",$F7&gt;=TODAY()-WEEKDAY(TODAY(),3),$F7&lt;=TODAY()-WEEKDAY(TODAY(),3)+6)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J7:J110">
+  <conditionalFormatting sqref="J7:J117">
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="7">
       <formula>"已完成"</formula>
     </cfRule>
@@ -7247,16 +7619,16 @@
       <formula>"延誤"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L7:L110">
+  <conditionalFormatting sqref="L7:L117">
     <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="5">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="J7:J110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="請從清單選擇：未開始、進行中、已完成、有風險、延誤" type="list">
+    <dataValidation sqref="J7:J117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" error="請從清單選擇：未開始、進行中、已完成、有風險、延誤" type="list">
       <formula1>"未開始,進行中,已完成,有風險,延誤"</formula1>
     </dataValidation>
-    <dataValidation sqref="K7:K110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
+    <dataValidation sqref="K7:K117" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -7359,11 +7731,29 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="n"/>
-      <c r="B4" s="10" t="n"/>
-      <c r="C4" s="10" t="n"/>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
+      <c r="A4" s="28" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>「Jacky 開發與測試」加入網頁 Wi-Fi 管理 7 項（R-37），W4 11/2–11/6</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>玩具連上 Wi-Fi 後沒有入口再加第二個；用戶要在網頁管理</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Jacky</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="28" t="n"/>

</xml_diff>